<commit_message>
Complete L2.4 NDT landscape and metric lessons with primary-source evidence
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,17 +567,17 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Soleymani, Baras, Hirche</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -585,215 +585,440 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Magazine</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>NDT / routing what-if</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/MCOM.001.2200012</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Polverini et al.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TNSM23:2038–2050</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>NDT / SDN conflict detection</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Soleymani, Baras, Hirche</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="72" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Paywall – cần thư viện</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="72" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Amad, van der Schaar</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D7" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>ICML 2026 (= P03)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Phương pháp</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>OA chưa tải</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2606.25923</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O4"/>
+  <autoFilter ref="A1:O7"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -801,7 +1026,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -814,7 +1044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -914,37 +1144,37 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -964,17 +1194,17 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>75 (S2, 2026-10-24)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -984,54 +1214,54 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1041,17 +1271,17 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>1 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1061,94 +1291,321 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>zhang2026opentwin</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: ranking loss, FQE.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>P/P/N</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Thứ cấp</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>amad2026dt2</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>L2.7 (Part 2b).</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O4"/>
+  <autoFilter ref="A1:O7"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1163,7 +1620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1190,120 +1647,132 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>3 nguồn giữ từ thư viện cũ; không phải danh sách đầy đủ về NDT, không là bài tập bắt buộc.</t>
+          <t>6 nguồn trong catalog hiện dùng; nguồn chính L2.4 ở đầu bảng. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Đọc chính NDT1 → P05 → P10. NMRG, P08, S07 chỉ tra bổ sung trong notes/literature/ndt_landscape.md, không thêm hàng đọc bắt buộc.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung trước dọn; các nhắc lesson/việc tiếp theo là lịch sử, không áp lịch học mới.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete L2.5 Part1 stale routing reading and verify illustrative examples
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,35 +567,35 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2022</v>
+        <v>2001</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -630,47 +630,47 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>NDT / routing what-if</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -698,36 +698,36 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/MCOM.001.2200012</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Polverini et al.</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -735,12 +735,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TNSM23:2038–2050</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -750,12 +750,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>NDT / SDN conflict detection</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -773,265 +773,342 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Có (local)</t>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>R34</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Kuri, Kumar</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>1995</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>IEEE TAC 40(8)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Journal</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>A6 Queue, thông tin trễ</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Chưa có xác nhận</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Paywall – cần thư viện</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>doi:10.1109/9.402238</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Kuri, Kumar</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TAC 40(8)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>A6 Queue, thông tin trễ</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Paywall – cần thư viện</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/9.402238</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Amad, van der Schaar</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D8" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>ICML 2026 (= P03)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Phương pháp</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>OA chưa tải</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2606.25923</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O7"/>
+  <autoFilter ref="A1:O8"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1044,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1144,42 +1221,42 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1194,17 +1271,17 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1214,44 +1291,44 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1271,17 +1348,17 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1298,37 +1375,37 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1346,15 +1423,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1371,37 +1452,37 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1419,19 +1500,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>75 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1441,54 +1518,54 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>LQG, CE tối ưu, không có clipping.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Chỉ trục state; không có trục model.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -1498,17 +1575,17 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>75 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>soleymani2022value</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1525,87 +1602,164 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: ranking loss, FQE.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>P/P/N</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Thứ cấp</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>amad2026dt2</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>L2.7 (Part 2b).</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O7"/>
+  <autoFilter ref="A1:O8"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1620,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1647,132 +1801,144 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>6 nguồn trong catalog hiện dùng; nguồn chính L2.4 ở đầu bảng. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>7 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Đọc chính NDT1 → P05 → P10. NMRG, P08, S07 chỉ tra bổ sung trong notes/literature/ndt_landscape.md, không thêm hàng đọc bắt buộc.</t>
+          <t>P04 ở đầu bảng: stale link-state, blocking và cost levels. M00/P01/Part2 chưa thực hiện; không tự ghi tác giả đã đọc.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete L2.5 Part2 reading and exact mechanism checks
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,45 +567,45 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2022</v>
+        <v>2001</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -705,47 +705,47 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>NDT / routing what-if</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -773,36 +773,36 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/MCOM.001.2200012</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Polverini et al.</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -810,12 +810,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TNSM23:2038–2050</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -825,12 +825,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>NDT / SDN conflict detection</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -848,252 +848,327 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Có (local)</t>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D7" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>R34</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Kuri, Kumar</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>1995</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>IEEE TAC 40(8)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Journal</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>A6 Queue, thông tin trễ</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Chưa có xác nhận</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Paywall – cần thư viện</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>doi:10.1109/9.402238</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Kuri, Kumar</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TAC 40(8)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>A6 Queue, thông tin trễ</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Paywall – cần thư viện</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/9.402238</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Amad, van der Schaar</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D9" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>ICML 2026 (= P03)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Phương pháp</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>OA chưa tải</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2606.25923</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O8"/>
+  <autoFilter ref="A1:O9"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1102,13 +1177,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1121,7 +1198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1221,37 +1298,37 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1266,22 +1343,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1298,42 +1375,42 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1348,17 +1425,17 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1368,44 +1445,44 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1425,17 +1502,17 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1452,37 +1529,37 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1500,15 +1577,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1525,37 +1606,37 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1573,19 +1654,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>75 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1595,54 +1672,54 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>LQG, CE tối ưu, không có clipping.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Chỉ trục state; không có trục model.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1652,17 +1729,17 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>75 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>soleymani2022value</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1679,87 +1756,164 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: ranking loss, FQE.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>P/P/N</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Thứ cấp</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>amad2026dt2</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>L2.7 (Part 2b).</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O8"/>
+  <autoFilter ref="A1:O9"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1774,7 +1928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1801,144 +1955,156 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>7 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>8 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>P04 ở đầu bảng: stale link-state, blocking và cost levels. M00/P01/Part2 chưa thực hiện; không tự ghi tác giả đã đọc.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen trong notes/literature/papers/P01.md, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete L2.6 Part A freshness and decision-value audit
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,45 +567,45 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2000</v>
+        <v>2026</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,62 +625,62 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (arxivv3 local,42trang)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,52 +700,52 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2022</v>
+        <v>2001</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -780,47 +780,47 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>NDT / routing what-if</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -848,36 +848,36 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/MCOM.001.2200012</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Polverini et al.</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -885,12 +885,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TNSM23:2038–2050</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>NDT / SDN conflict detection</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -923,252 +923,327 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>Có (local)</t>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D8" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="72" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>R34</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Kuri, Kumar</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>1995</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>IEEE TAC 40(8)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Journal</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>A6 Queue, thông tin trễ</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Chưa có xác nhận</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Paywall – cần thư viện</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>doi:10.1109/9.402238</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Kuri, Kumar</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TAC 40(8)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>A6 Queue, thông tin trễ</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Paywall – cần thư viện</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/9.402238</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Amad, van der Schaar</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D10" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>ICML 2026 (= P03)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Phương pháp</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>OA chưa tải</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2606.25923</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O9"/>
+  <autoFilter ref="A1:O10"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1179,13 +1254,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1198,7 +1275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1298,37 +1375,37 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1343,22 +1420,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1375,37 +1452,37 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1420,22 +1497,22 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1452,42 +1529,42 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1502,17 +1579,17 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1522,44 +1599,44 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1579,17 +1656,17 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1606,37 +1683,37 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1654,15 +1731,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1679,37 +1760,37 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1727,19 +1808,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>75 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1749,54 +1826,54 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>LQG, CE tối ưu, không có clipping.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Chỉ trục state; không có trục model.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1806,17 +1883,17 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>75 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>soleymani2022value</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1833,87 +1910,164 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: ranking loss, FQE.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>P/P/N</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Thứ cấp</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>amad2026dt2</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>L2.7 (Part 2b).</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O9"/>
+  <autoFilter ref="A1:O10"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1928,7 +2082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1955,156 +2109,168 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>8 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>9 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen trong notes/literature/papers/P01.md, chưa cần đọc full.</t>
+          <t>S11 hiện tại: freshness → decision cost; bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; P13/Part B, tác giả L-self/Gate còn mở.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete L2.6 Part B transient horizon checks and boundary
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,45 +567,45 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2026</v>
+        <v>2017</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,62 +625,62 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2000</v>
+        <v>2026</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,62 +700,62 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (arxivv3 local,42trang)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -775,52 +775,52 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2022</v>
+        <v>2001</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -855,47 +855,47 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>NDT / routing what-if</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -923,36 +923,36 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/MCOM.001.2200012</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Polverini et al.</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -960,12 +960,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TNSM23:2038–2050</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -975,12 +975,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>NDT / SDN conflict detection</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -998,252 +998,327 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Có (local)</t>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D9" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>R34</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Kuri, Kumar</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>1995</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>IEEE TAC 40(8)</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Journal</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>A6 Queue, thông tin trễ</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Chưa có xác nhận</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Paywall – cần thư viện</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>doi:10.1109/9.402238</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Kuri, Kumar</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TAC 40(8)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>A6 Queue, thông tin trễ</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Paywall – cần thư viện</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/9.402238</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Amad, van der Schaar</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D11" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>ICML 2026 (= P03)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Phương pháp</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>OA chưa tải</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2606.25923</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O10"/>
+  <autoFilter ref="A1:O11"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1256,13 +1331,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1275,7 +1352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1375,42 +1452,42 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1425,17 +1502,17 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>1 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1452,37 +1529,37 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1497,22 +1574,22 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1529,37 +1606,37 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1574,22 +1651,22 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1606,42 +1683,42 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1656,17 +1733,17 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1676,44 +1753,44 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1733,17 +1810,17 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1760,37 +1837,37 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1808,15 +1885,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1833,37 +1914,37 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1881,19 +1962,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>75 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1903,54 +1980,54 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>LQG, CE tối ưu, không có clipping.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Chỉ trục state; không có trục model.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1960,17 +2037,17 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>75 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>soleymani2022value</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1987,87 +2064,164 @@
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>R51</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>DT2: Decision-Targeted Digital Twins</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: ranking loss, FQE.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>P/P/N</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Thứ cấp</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>amad2026dt2</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>L2.7 (Part 2b).</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O10"/>
+  <autoFilter ref="A1:O11"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2082,7 +2236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2109,168 +2263,180 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>9 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>10 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>S11 hiện tại: freshness → decision cost; bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; P13/Part B, tác giả L-self/Gate còn mở.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B15"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Document L2.7 Part A fidelity and oracle evidence; mark P02 full-text blocked
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,35 +567,35 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Britt Mathijsen; Bert Zwart</t>
+          <t>Harry Amad; Mihaela van der Schaar</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2017</v>
+        <v>2026</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Queueing Systems85(3–4):269–304</t>
+          <t>ICML2026, PMLR306:2207–2233</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Journal (đọc VoR CWI)</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Lý thuyết / numerical study</t>
+          <t>Phương pháp</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Queueing / transient approximation / staffing</t>
+          <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
+          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,62 +625,62 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (journal36trang local)</t>
+          <t>Có (PMLR27trang local)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s11134-016-9511-0</t>
+          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
+          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>USENIX NSDI23:1557–1581</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Phương pháp / empirical TE</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>WAN traffic engineering / direct optimization</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,72 +700,72 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (USENIX26trang gồm cover)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2000</v>
+        <v>2023</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>TR-C153:104174</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Journal (full text chưa lấy được)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Sensitivity / predictive control</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Control methodology / nguồn tác giả chỉ định</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -773,54 +773,54 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Có (submission28trang local)</t>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED full text; OA record CC BY</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>doi:10.1016/j.trc.2023.104174</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2001</v>
+        <v>2017</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -850,62 +850,62 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -925,62 +925,62 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (arxivv3 local,42trang)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2026</v>
+        <v>2000</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -998,64 +998,64 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2026</v>
+        <v>2001</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1080,29 +1080,29 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Soleymani, Baras, Hirche</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -1110,215 +1110,365 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Magazine</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>NDT / routing what-if</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/MCOM.001.2200012</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Polverini et al.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TNSM23:2038–2050</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>NDT / SDN conflict detection</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Soleymani, Baras, Hirche</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="72" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D13" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Paywall – cần thư viện</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>R51</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>DT2: Decision-Targeted Digital Twins</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Amad, van der Schaar</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>ICML 2026 (= P03)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Conference</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Phương pháp</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>A1/A5 Decision-targeted twin</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>• Model trung bình M0 đủ tốt ở M19–M22 nhưng không đủ ở M01–M04</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Chưa có xác nhận</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>OA chưa tải</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2606.25923</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>Cầu nối phương pháp DT; không phải paper NDT/networking chuyên biệt. R51 = P03.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O11"/>
+  <autoFilter ref="A1:O13"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1327,19 +1477,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1352,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1452,42 +1606,42 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
+          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
+          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
+          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
+          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
+          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>N/P/N</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1497,22 +1651,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Có link §2/PDF2; chưa chạy</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-26)</t>
+          <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>mathijsen2017transient</t>
+          <t>amad2026dt2</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
+          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1529,42 +1683,42 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Tối ưu TE khi future demand khó dự đoán.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1574,22 +1728,22 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Có link §4.1; chưa chạy</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>perry2023dote</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1606,67 +1760,67 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa kiểm</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>4 (Crossref,2026-10-26)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>poelman2023structurefree</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1683,42 +1837,42 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1728,22 +1882,22 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>1 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1760,42 +1914,42 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1805,22 +1959,22 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1830,49 +1984,49 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1882,22 +2036,22 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1907,49 +2061,49 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1962,15 +2116,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>117 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1980,44 +2138,44 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -2037,17 +2195,17 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>75 (S2, 2026-10-24)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2057,54 +2215,54 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>R34</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Chưa đánh giá.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>P/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Metadata</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -2114,17 +2272,17 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>34 (Crossref, 2026-10-24)</t>
+          <t>1 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>kuri1995optimal</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -2134,44 +2292,44 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DT2: Decision-Targeted Digital Twins</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Theo Final Review: huấn luyện digital twin để chọn policy tốt.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Theo Final Review: ranking loss, FQE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Lượt này chỉ trích dẫn xuôi; nội dung theo Final Review §3.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Theo Final Review: Theorem 3.1 là mệnh đề tồn tại.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Dự án không huấn luyện model; đo giá trị law đúng so với xấp xỉ trung bình.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2181,7 +2339,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Thứ cấp</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2189,19 +2347,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>1 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>amad2026dt2</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>L2.7 (Part 2b).</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -2211,17 +2365,171 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
+    <row r="13" ht="84" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Optimal control of arrivals to queues with delayed queue length information</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đọc.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa đánh giá.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>P/P/P</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>34 (Crossref, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>kuri1995optimal</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6).</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O11"/>
+  <autoFilter ref="A1:O13"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2236,7 +2544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2263,180 +2571,192 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>12 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 chưa thực hiện. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DT² là cầu nối phương pháp digital twin, không phải paper networking chuyên biệt.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete L2.7 Part B VE and operational regret-equivalence artifacts
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,35 +567,35 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Harry Amad; Mihaela van der Schaar</t>
+          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2026</v>
+        <v>2020</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ICML2026, PMLR306:2207–2233</t>
+          <t>NeurIPS33</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp</t>
+          <t>Khái niệm / model-based RL</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>A1/A5 Decision-targeted twin</t>
+          <t>Value equivalence / decision-relevant models</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
+          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,52 +625,52 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (PMLR27trang local)</t>
+          <t>Có (NeurIPS12trang local)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
+          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
+          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
+          <t>Harry Amad; Mihaela van der Schaar</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>USENIX NSDI23:1557–1581</t>
+          <t>ICML2026, PMLR306:2207–2233</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp / empirical TE</t>
+          <t>Phương pháp</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>WAN traffic engineering / direct optimization</t>
+          <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
+          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,34 +700,34 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (USENIX26trang gồm cover)</t>
+          <t>Có (PMLR27trang local)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
+          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
+          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
+          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -735,17 +735,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TR-C153:104174</t>
+          <t>USENIX NSDI23:1557–1581</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Journal (full text chưa lấy được)</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity / predictive control</t>
+          <t>Phương pháp / empirical TE</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -755,17 +755,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Control methodology / nguồn tác giả chỉ định</t>
+          <t>WAN traffic engineering / direct optimization</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
+          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -773,54 +773,54 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED full text; OA record CC BY</t>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Có (USENIX26trang gồm cover)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1016/j.trc.2023.104174</t>
+          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
+          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Britt Mathijsen; Bert Zwart</t>
+          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2017</v>
+        <v>2023</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Queueing Systems85(3–4):269–304</t>
+          <t>TR-C153:104174</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Journal (đọc VoR CWI)</t>
+          <t>Journal (full text chưa lấy được)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Lý thuyết / numerical study</t>
+          <t>Sensitivity / predictive control</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Queueing / transient approximation / staffing</t>
+          <t>Control methodology / nguồn tác giả chỉ định</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
+          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -848,64 +848,64 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Có (journal36trang local)</t>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>BLOCKED full text; OA record CC BY</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s11134-016-9511-0</t>
+          <t>doi:10.1016/j.trc.2023.104174</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
+          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2026</v>
+        <v>2017</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -925,62 +925,62 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2000</v>
+        <v>2026</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1000,62 +1000,62 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (arxivv3 local,42trang)</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2001</v>
+        <v>2000</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1075,52 +1075,52 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2022</v>
+        <v>2001</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1155,47 +1155,47 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Survey</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>NDT / routing what-if</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1223,36 +1223,36 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/MCOM.001.2200012</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Polverini et al.</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -1260,12 +1260,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TNSM23:2038–2050</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>NDT / SDN conflict detection</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1298,177 +1298,252 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Có (local)</t>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D13" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="72" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D14" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Paywall – cần thư viện</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O13"/>
+  <autoFilter ref="A1:O14"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1477,8 +1552,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
@@ -1488,12 +1563,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1506,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1606,37 +1683,37 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
+          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
+          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
+          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
+          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
+          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1651,22 +1728,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Có link §2/PDF2; chưa chạy</t>
+          <t>Chưa kiểm/chạy paper code</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>1 (S2, 2026-10-24)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>amad2026dt2</t>
+          <t>grimm2020valueequivalence</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
+          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1683,37 +1760,37 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tối ưu TE khi future demand khó dự đoán.</t>
+          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
+          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
+          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
+          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
+          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1728,22 +1805,22 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Có link §4.1; chưa chạy</t>
+          <t>Có link §2/PDF2; chưa chạy</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>perry2023dote</t>
+          <t>amad2026dt2</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
+          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1760,37 +1837,37 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
+          <t>Tối ưu TE khi future demand khó dự đoán.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
+          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
+          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
+          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
+          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1800,27 +1877,27 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Có link §4.1; chưa chạy</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>4 (Crossref,2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>poelman2023structurefree</t>
+          <t>perry2023dote</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
+          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1837,67 +1914,67 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
+          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
+          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
+          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
+          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
+          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>N/P/N</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Chưa kiểm</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-26)</t>
+          <t>4 (Crossref,2026-10-26)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>mathijsen2017transient</t>
+          <t>poelman2023structurefree</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
+          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1914,42 +1991,42 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1964,17 +2041,17 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>1 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1991,37 +2068,37 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -2036,22 +2113,22 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2068,37 +2145,37 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -2113,22 +2190,22 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2145,42 +2222,42 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -2195,17 +2272,17 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2215,44 +2292,44 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -2272,17 +2349,17 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -2299,37 +2376,37 @@
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2347,15 +2424,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>polverini2026conflicts</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -2372,37 +2453,37 @@
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -2420,19 +2501,15 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>75 (S2, 2026-10-24)</t>
-        </is>
-      </c>
+      <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>zhang2026opentwin</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -2442,94 +2519,171 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="84" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Chưa đánh giá.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>P/P/P</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Metadata</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>34 (Crossref, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>kuri1995optimal</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Part 2b (L2.6).</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O13"/>
+  <autoFilter ref="A1:O14"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2544,7 +2698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2571,192 +2725,204 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>12 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>13 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part A</t>
+          <t>L2.7 Part B</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 chưa thực hiện. Không tự cấp L-self/Gate.</t>
+          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 chưa thực hiện. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete targeted L2.8 reading and replay Cooper allocation example
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,45 +567,45 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
+          <t>Akram Almohammedi; Mohammed Balfaqih; Sam Darshi; Rami Langar; Wael Jaafar</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>NeurIPS33</t>
+          <t>arXiv2607.22857v1; submitted TNSM</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Khái niệm / model-based RL</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Value equivalence / decision-relevant models</t>
+          <t>NDT/networking</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
+          <t>PC3/PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,34 +625,34 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (NeurIPS12trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
+          <t>https://arxiv.org/abs/2607.22857v1</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Harry Amad; Mihaela van der Schaar</t>
+          <t>Rui Min; Xianyao Li; Fang Xu; Eric Jing Du (metadata: Jing Du)</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -660,27 +660,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>ICML2026, PMLR306:2207–2233</t>
+          <t>arXiv2610.05550v1</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Preprint under review</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>A1/A5 Decision-targeted twin</t>
+          <t>World model/repair diagnosis</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
+          <t>PC3/PC4; Tier1 framing AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,52 +700,52 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (PMLR27trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
+          <t>https://arxiv.org/abs/2610.05550v1</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
+          <t>L2.8 Part2: Tier1 framing; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
+          <t>Jayakumar Subramanian; Amit Sinha; Raihan Seraj; Aditya Mahajan</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>USENIX NSDI23:1557–1581</t>
+          <t>JMLR23(12):1–83</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp / empirical TE</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -755,17 +755,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>WAN traffic engineering / direct optimization</t>
+          <t>Partial observations/model adequacy</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
+          <t>PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -775,52 +775,52 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Có (USENIX26trang gồm cover)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
+          <t>https://www.jmlr.org/papers/v23/20-1165.html</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
+          <t>Nicola Secomandi</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2023</v>
+        <v>2008</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TR-C153:104174</t>
+          <t>MSOM10(3):468–483</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Journal (full text chưa lấy được)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity / predictive control</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Control methodology / nguồn tác giả chỉ định</t>
+          <t>RM/conditions</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -848,54 +848,54 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED full text; OA record CC BY</t>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1016/j.trc.2023.104174</t>
+          <t>doi:10.1287/msom.1070.0184</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Britt Mathijsen; Bert Zwart</t>
+          <t>William L. Cooper</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2017</v>
+        <v>2002</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Queueing Systems85(3–4):269–304</t>
+          <t>Operations Research50(4):720–727</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Journal (đọc VoR CWI)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Lý thuyết / numerical study</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -905,17 +905,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Queueing / transient approximation / staffing</t>
+          <t>RM/negative information value</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
+          <t>PC3; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -925,72 +925,72 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Có (journal36trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s11134-016-9511-0</t>
+          <t>doi:10.1287/opre.50.4.720.2855</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Lijian Chen; Tito Homem-de-Mello</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2026</v>
+        <v>2010</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>Annals OR177:91–114; online2009</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Journal; đọc TR2006</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có (journal)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>RM/non-deterioration</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1000,62 +1000,62 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>doi:10.1007/s10479-009-0603-7</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2000</v>
+        <v>2020</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>NeurIPS33</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Khái niệm / model-based RL</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Value equivalence / decision-relevant models</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1075,52 +1075,52 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (NeurIPS12trang local)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Harry Amad; Mihaela van der Schaar</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2001</v>
+        <v>2026</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>ICML2026, PMLR306:2207–2233</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Phương pháp</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1150,52 +1150,52 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (PMLR27trang local)</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>USENIX NSDI23:1557–1581</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Phương pháp / empirical TE</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>WAN traffic engineering / direct optimization</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1225,52 +1225,52 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (USENIX26trang gồm cover)</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>TR-C153:104174</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal (full text chưa lấy được)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Sensitivity / predictive control</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>Control methodology / nguồn tác giả chỉ định</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1300,62 +1300,62 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Full text web; PDF local403</t>
+          <t>BLOCKED full text; OA record CC BY</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1016/j.trc.2023.104174</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2026</v>
+        <v>2017</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1375,175 +1375,625 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TIT72(4):2237–2276</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Journal; đọc arxivv3</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Mô hình / tối ưu</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Có (identity đã kiểm)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Networking / goal-oriented remote decisions</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Có (arxivv3 local,42trang)</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TIT.2026.3663678</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>M00</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>How Useful Is Old Information?</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Michael Mitzenmacher</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TPDS11(1):6–20</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Journal; PDF là submission</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Mô hình / simulation</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Có (journal identity)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Networking / load balancing, stale queues</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Có (submission28trang local)</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/71.824633</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Shaikh, Rexford, Shin</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>IEEE/ACM ToN9(2):162–176</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Thực nghiệm / đánh giá</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>QoS routing / stale link-state</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/90.917073</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>NDT1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Almasan et al.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Magazine</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>NDT / routing what-if</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/MCOM.001.2200012</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Polverini et al.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TNSM23:2038–2050</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>NDT / SDN conflict detection</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D19" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="72" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D20" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Paywall – cần thư viện</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O14"/>
+  <autoFilter ref="A1:O20"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1554,23 +2004,35 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1583,7 +2045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1683,37 +2145,37 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
+          <t>NDT gate/utility regret trong networking đã có.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
+          <t>EWMA on-policy error + live-validated fallback.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
+          <t>§III–VI/PDF5–9: utility regret, feedback gate, injected neighbor-power offset.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
+          <t>Chưa chạy MATLAB; threshold chọn trên evaluation runs.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
+          <t>Không D20×D21; 21 power blends, khác one-shot queue.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1728,22 +2190,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm/chạy paper code</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>grimm2020valueequivalence</t>
+          <t>almohammedi2026twinfidelity</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -1760,37 +2222,37 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
+          <t>Sửa phần lỗi lớn nhất có cho action tốt nhất?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
+          <t>Matched-candidate center/response P,C,S,E grid.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
+          <t>§4–5/F.1 Eq10/PDF4–5,22: 2×2 repair; §7.1/F.2: MSE/decision inversion.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
+          <t>True-future diagnostic oracles có unequal info budgets; chưa chạy experiments.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
+          <t>Center qua action pool không D20; E không D15 true oracle.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1805,22 +2267,22 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Có link §2/PDF2; chưa chạy</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>1 (S2, 2026-10-24)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>amad2026dt2</t>
+          <t>min2026misleads</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -1837,37 +2299,37 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Tối ưu TE khi future demand khó dự đoán.</t>
+          <t>Thông tin/model cần giữ gì để planning đủ tốt?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
+          <t>History compression + reward/transition approximation.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
+          <t>Def3/7,Thm5/9/PDF6–8,15–18: policy loss≤2αt.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
+          <t>Uniform reward/IPM bounds; không full83pages hoặc chạy code.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
+          <t>Không independent D20×D21 hoặc GM/Cref; chưa chứng nhận bound cho plant.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1882,22 +2344,22 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Có link §4.1; chưa chạy</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>perry2023dote</t>
+          <t>subramanian2022ais</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1914,37 +2376,37 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
+          <t>Điều kiện đủ để re-solving không làm hại?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
+          <t>Sequential consistency + policy-objective accuracy.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
+          <t>§3 Def2–5/Props1–3/PDF8–10: SC+Π-accuracy⇒SI⇒non-deterioration.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
+          <t>α bounds thường cần policy evaluation; chưa là usable predictive H1.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
+          <t>MP-feasibility khác action-feasibility; plant mapping là sufficient diagnostic.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1954,27 +2416,27 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>4 (Crossref,2026-10-26)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>poelman2023structurefree</t>
+          <t>secomandi2008resolving</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1991,42 +2453,42 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
+          <t>Cập nhật allocation có thể hại?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
+          <t>DLP re-solve theo capacity/conditional demand.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
+          <t>§5 Example1/Eq10/PDF7: conditional revenue8.96→7.59; own full-expectation replay14.586589→14.079588.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
+          <t>Không rounding; không full asymptotic proofs/Phase3 hoặc RM four-cell replication.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
+          <t>Multi-step booking khác one-shot queue; CE không cùng Jensen mechanism.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>N/P/N</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2036,22 +2498,22 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>R02 Example1 analytic replay</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>mathijsen2017transient</t>
+          <t>cooper2002asymptotic</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -2068,42 +2530,42 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Vì sao SLP allocation re-solve không hại?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Integer allocation; objective bằng true policy expected revenue.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>TR Prop1/PDF10–11; §4/PDF16 bid-price có thể hại dù từ SLP.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>Journal proposition numbering chưa kiểm; không mọi policy/true MDP.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Cùng proof structure K-S8, khác literal EVPPI và D20 intervention.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -2113,22 +2575,22 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>chen2010resolving</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2145,42 +2607,42 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -2190,22 +2652,22 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa kiểm/chạy paper code</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>grimm2020valueequivalence</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2222,42 +2684,42 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -2267,22 +2729,22 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Có link §2/PDF2; chưa chạy</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>amad2026dt2</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2299,37 +2761,37 @@
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Tối ưu TE khi future demand khó dự đoán.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -2344,22 +2806,22 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Có link §4.1; chưa chạy</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>perry2023dote</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -2369,44 +2831,44 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2416,7 +2878,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2426,17 +2888,17 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>4 (Crossref,2026-10-26)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>poelman2023structurefree</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -2446,49 +2908,49 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2498,18 +2960,22 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="n"/>
+          <t>Chưa chạy code paper</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -2519,49 +2985,49 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -2571,22 +3037,22 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>75 (S2, 2026-10-24)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -2596,94 +3062,552 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>M00</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>How Useful Is Old Information?</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>N/P/P</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm code nguồn paper</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>128 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>mitzenmacher2000oldinfo</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="84" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>N/P/P</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>117 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>shaikh2001stale</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>NDT1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>185 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>almasan2022ndt</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="84" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>polverini2026conflicts</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="84" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>zhang2026opentwin</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="84" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="84" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Chưa đánh giá.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>P/P/P</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Metadata</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>34 (Crossref, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>kuri1995optimal</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Part 2b (L2.6).</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O14"/>
+  <autoFilter ref="A1:O20"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2698,7 +3622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2725,204 +3649,216 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>13 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>19 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part B</t>
+          <t>L2.8 Part2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
+          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part A</t>
+          <t>L2.7 Part B</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 chưa thực hiện. Không tự cấp L-self/Gate.</t>
+          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B18"/>
+  <autoFilter ref="A1:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Read P02 VoR, add raw-captured L2.8 follow-up search and screen pending proposals
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Journal (full text chưa lấy được)</t>
+          <t>Journal (VoR, CC BY)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC5: errors, horizon/update; chưa kiểm factorial hoặc dấu Γ.</t>
+          <t>• PC2 (PHASE_2 v2.0 §5.4: nguồn quyết định nhãn) / PC3/PC4/PC5: bias một đại lượng mỗi lần; sweep 1-D theo prediction/update horizon; không gán dấu Γ.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1298,9 +1298,9 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>BLOCKED full text; OA record CC BY</t>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>Có (VoR 20 trang local; tác giả tải 26/10)</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: abstract-only, §2–4/hình còn mở; không tự ghi T.</t>
+          <t>L2.7 PartA dependency: AI-T VoR §1–5 + Bảng 2 (L2.8 follow-up 26/10); chưa L-self.</t>
         </is>
       </c>
     </row>
@@ -2016,23 +2016,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -2853,17 +2854,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Abstract: simulator, model/input aggregation+bias, horizon và update frequency.</t>
+          <t>Aimsun + MPC structure-free 4 nút; I reference biết demand ghi sẵn → II aggregation → III bias trên aggregation (§2.1, §2.2.4).</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Official abstract: update thường hơn dampens errors; không xác nhận các số trong lesson.</t>
+          <t>Bias 1 đại lượng/lần (§3.3.1 tr15); Bảng 2 tr16 quét prediction 12/30/60 s và update 12/30/60 s; update ngắn bù một phần, state bias lớn làm mất bù (§3.3.2, §4).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Full text timeout/403; OAT/joint-bias và recorded-future comparator chưa kiểm.</t>
+          <t>Không joint bias (§4 tr18); solver heuristic &lt;1% so full B&amp;B (Fig3d); metric delay/xe so reference, không regret/oracle D15. Hình chỉ đọc caption.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2878,7 +2879,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2898,7 +2899,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Đọc VoR §2.1/2.2.4/3/4 và captions khi truy cập được; MT2/6/7 chưa đóng.</t>
+          <t>Tác giả đọc §2.2.4, §3.3, Bảng 2 nếu dùng cho nhãn PC2 ở L2.9; MT2/6/7 cập nhật ở follow-up.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -3622,7 +3623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -3656,209 +3657,221 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2</t>
+          <t>L2.8 follow-up</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
+          <t>26/10: P02 nay có VoR do bạn tải; AI-T §1–5 + Bảng 2: bias một đại lượng mỗi lần, quét 1-D theo prediction/update horizon, không joint bias. Phiên tìm bổ sung lưu raw response; 3 đề xuất mới và 6 đề xuất cũ đã sàng abstract, chờ duyệt, chưa thêm hàng. Không L2.9/Gate.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part B</t>
+          <t>L2.8 Part2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
+          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part A</t>
+          <t>L2.7 Part B</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
+          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Read approved IA26, DTS25, CEN26 and CEH23; add to library and confirm provisional labels unchanged
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,11 +12,11 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,17 +567,17 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NDT26</t>
+          <t>IA26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
+          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Akram Almohammedi; Mohammed Balfaqih; Sam Darshi; Rami Langar; Wael Jaafar</t>
+          <t>Scott Moeller; Bhaskar Krishnamachari</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -585,7 +585,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>arXiv2607.22857v1; submitted TNSM</t>
+          <t>arXiv2609.06351v1</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Theory / networked decisions</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>NDT/networking</t>
+          <t>Networking/control: freshness × scope</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
+          <t>• PC2/PC6: giá trị thông tin hiện tại theo decision-relevant predictability; môi trường ngoại sinh.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,72 +625,72 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2607.22857v1</t>
+          <t>https://arxiv.org/abs/2609.06351v1</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-T §1–2.3, §3.4; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>WM26</t>
+          <t>DTS25</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
+          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Rui Min; Xianyao Li; Fang Xu; Eric Jing Du (metadata: Jing Du)</t>
+          <t>Zhiheng Yang; Francisco Vogt; Adam Belloum; Christian Rothenberg; Paola Grosso; Chrysa Papagianni</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>arXiv2610.05550v1</t>
+          <t>CoNEXT'25 Student Workshop</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Preprint under review</t>
+          <t>Workshop (2 trang)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Vision / NDT sync</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác nhận</t>
+          <t>Workshop sinh viên</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>World model/repair diagnosis</t>
+          <t>NDT/networking</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 framing AI đề xuất, không đổi nhãn.</t>
+          <t>• PC2/PC6 framing: chọn telemetry theo giá trị quyết định; chưa có thí nghiệm.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -700,72 +700,72 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2610.05550v1</t>
+          <t>doi:10.1145/3769700.3771695</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 framing; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-F 2 trang; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AIS22</t>
+          <t>CEN26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
+          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Jayakumar Subramanian; Amit Sinha; Raihan Seraj; Aditya Mahajan</t>
+          <t>Zifan Zhang; Zhichao Hou; Tingxiang Ji; Yuchen Liu</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>JMLR23(12):1–83</t>
+          <t>arXiv2608.01725v1</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Telemetry model / decision replay</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Partial observations/model adequacy</t>
+          <t>Networking/systems telemetry</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Tra khi cần</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
+          <t>• PC5: đánh giá model bằng quyết định replay; không 2×2.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -775,62 +775,62 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>https://www.jmlr.org/papers/v23/20-1165.html</t>
+          <t>https://arxiv.org/abs/2608.01725v1</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-T §I, §III-D, §IV-A, §IV-D; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>CEH23</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
+          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nicola Secomandi</t>
+          <t>Chen Yan; Alexandre Reiffers-Masson</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2008</v>
+        <v>2023</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>MSOM10(3):468–483</t>
+          <t>arXiv2308.13166v1; submitted to Operations Research</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Stochastic optimization / CE bounds</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>RM/conditions</t>
+          <t>OR / certainty equivalence</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>• PC5/PC3: cận khoảng cách CE–tối ưu ∝√var hoặc var; cần động học affine trong kỳ vọng.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -850,47 +850,47 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1287/msom.1070.0184</t>
+          <t>https://arxiv.org/abs/2308.13166v1</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-T §2, §5.1, §6.1–6.3, §8; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>William L. Cooper</t>
+          <t>Akram Almohammedi; Mohammed Balfaqih; Sam Darshi; Rami Langar; Wael Jaafar</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2002</v>
+        <v>2026</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Operations Research50(4):720–727</t>
+          <t>arXiv2607.22857v1; submitted TNSM</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -900,22 +900,22 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>RM/negative information value</t>
+          <t>NDT/networking</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Tra khi cần</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>PC3; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>PC3/PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -930,42 +930,42 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1287/opre.50.4.720.2855</t>
+          <t>https://arxiv.org/abs/2607.22857v1</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Re-solving stochastic programming models for airline revenue management</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Lijian Chen; Tito Homem-de-Mello</t>
+          <t>Rui Min; Xianyao Li; Fang Xu; Eric Jing Du (metadata: Jing Du)</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2010</v>
+        <v>2026</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Annals OR177:91–114; online2009</t>
+          <t>arXiv2610.05550v1</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc TR2006</t>
+          <t>Preprint under review</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -975,22 +975,22 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Có (journal)</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>RM/non-deterioration</t>
+          <t>World model/repair diagnosis</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Tra khi cần</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>PC3/PC4; Tier1 framing AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1005,47 +1005,47 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s10479-009-0603-7</t>
+          <t>https://arxiv.org/abs/2610.05550v1</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>L2.8 Part2: Tier1 framing; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
+          <t>Jayakumar Subramanian; Amit Sinha; Raihan Seraj; Aditya Mahajan</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>NeurIPS33</t>
+          <t>JMLR23(12):1–83</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Khái niệm / model-based RL</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1055,17 +1055,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Value equivalence / decision-relevant models</t>
+          <t>Partial observations/model adequacy</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
+          <t>PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1075,52 +1075,52 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Có (NeurIPS12trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
+          <t>https://www.jmlr.org/papers/v23/20-1165.html</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Harry Amad; Mihaela van der Schaar</t>
+          <t>Nicola Secomandi</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2026</v>
+        <v>2008</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ICML2026, PMLR306:2207–2233</t>
+          <t>MSOM10(3):468–483</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>A1/A5 Decision-targeted twin</t>
+          <t>RM/conditions</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1150,52 +1150,52 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Có (PMLR27trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
+          <t>doi:10.1287/msom.1070.0184</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
+          <t>William L. Cooper</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2023</v>
+        <v>2002</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>USENIX NSDI23:1557–1581</t>
+          <t>Operations Research50(4):720–727</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp / empirical TE</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1205,17 +1205,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>WAN traffic engineering / direct optimization</t>
+          <t>RM/negative information value</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
+          <t>PC3; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1225,72 +1225,72 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Có (USENIX26trang gồm cover)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
+          <t>doi:10.1287/opre.50.4.720.2855</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
+          <t>Lijian Chen; Tito Homem-de-Mello</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2023</v>
+        <v>2010</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TR-C153:104174</t>
+          <t>Annals OR177:91–114; online2009</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Journal (VoR, CC BY)</t>
+          <t>Journal; đọc TR2006</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity / predictive control</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Control methodology / nguồn tác giả chỉ định</t>
+          <t>RM/non-deterioration</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>• PC2 (PHASE_2 v2.0 §5.4: nguồn quyết định nhãn) / PC3/PC4/PC5: bias một đại lượng mỗi lần; sweep 1-D theo prediction/update horizon; không gán dấu Γ.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1300,52 +1300,52 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Có (VoR 20 trang local; tác giả tải 26/10)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1016/j.trc.2023.104174</t>
+          <t>doi:10.1007/s10479-009-0603-7</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA dependency: AI-T VoR §1–5 + Bảng 2 (L2.8 follow-up 26/10); chưa L-self.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Britt Mathijsen; Bert Zwart</t>
+          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Queueing Systems85(3–4):269–304</t>
+          <t>NeurIPS33</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Journal (đọc VoR CWI)</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Lý thuyết / numerical study</t>
+          <t>Khái niệm / model-based RL</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Queueing / transient approximation / staffing</t>
+          <t>Value equivalence / decision-relevant models</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
+          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1375,34 +1375,34 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Có (journal36trang local)</t>
+          <t>Có (NeurIPS12trang local)</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s11134-016-9511-0</t>
+          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
+          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Harry Amad; Mihaela van der Schaar</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -1410,27 +1410,27 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>ICML2026, PMLR306:2207–2233</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Phương pháp</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1450,62 +1450,62 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (PMLR27trang local)</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2000</v>
+        <v>2023</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>USENIX NSDI23:1557–1581</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Phương pháp / empirical TE</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>WAN traffic engineering / direct optimization</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1525,52 +1525,52 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (USENIX26trang gồm cover)</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="72" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2001</v>
+        <v>2023</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>TR-C153:104174</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal (VoR, CC BY)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Sensitivity / predictive control</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1580,17 +1580,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Control methodology / nguồn tác giả chỉ định</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC2 (PHASE_2 v2.0 §5.4: nguồn quyết định nhãn) / PC3/PC4/PC5: bias một đại lượng mỗi lần; sweep 1-D theo prediction/update horizon; không gán dấu Γ.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1600,52 +1600,52 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (VoR 20 trang local; tác giả tải 26/10)</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1016/j.trc.2023.104174</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.7 PartA dependency: AI-T VoR §1–5 + Bảng 2 (L2.8 follow-up 26/10); chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="72" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1675,34 +1675,34 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="72" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -1710,27 +1710,27 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1748,64 +1748,64 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Có (arxivv3 local,42trang)</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="72" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2026</v>
+        <v>2000</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1825,175 +1825,475 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="72" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Shaikh, Rexford, Shin</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>IEEE/ACM ToN9(2):162–176</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Thực nghiệm / đánh giá</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>QoS routing / stale link-state</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/90.917073</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>NDT1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Almasan et al.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Magazine</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>NDT / routing what-if</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/MCOM.001.2200012</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Polverini et al.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TNSM23:2038–2050</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>NDT / SDN conflict detection</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Value of Information in Feedback Control: Quantification</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Soleymani, Baras, Hirche</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D23" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="M23" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="72" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D24" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Paywall – cần thư viện</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O20"/>
+  <autoFilter ref="A1:O24"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2028,12 +2328,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -2046,7 +2354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2146,42 +2454,42 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NDT26</t>
+          <t>IA26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
+          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>NDT gate/utility regret trong networking đã có.</t>
+          <t>Thông tin mới-cục bộ hay đầy đủ-trễ cho quyết định đội?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>EWMA on-policy error + live-validated fallback.</t>
+          <t>Cost bậc hai, x*=Q⁻¹b(θ_t); regret so thông tin hiện tại đầy đủ (§2.3 Eq19–21).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>§III–VI/PDF5–9: utility regret, feedback gate, injected neighbor-power offset.</t>
+          <t>Định lý 3 §3.4 tr13–14: fresh-local thắng ⇔ τ/T &gt; ½log(1/(1−η_S(0))); Eq22–23: thêm thông tin cùng độ tươi không hại.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy MATLAB; threshold chọn trên evaluation runs.</t>
+          <t>Môi trường không bị action điều khiển; loại trừ controlled queueing (§1 tr3).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Không D20×D21; 21 power blends, khác one-shot queue.</t>
+          <t>Không trục model, không Γ; repo là quyết định làm đổi tải có mode ẩn.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>P/N/N</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2191,22 +2499,18 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>almohammedi2026twinfidelity</t>
+          <t>ia26</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Tác giả đọc §2.3, §3.4 nếu dùng cho PC6.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -2223,67 +2527,63 @@
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>WM26</t>
+          <t>DTS25</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
+          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Sửa phần lỗi lớn nhất có cho action tốt nhất?</t>
+          <t>Đo gì, ở đâu, khi nào để đồng bộ NDT dưới ngân sách?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Matched-candidate center/response P,C,S,E grid.</t>
+          <t>Neural Measurement Field λθ(e,t,f,p|z_c) học online (§2).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>§4–5/F.1 Eq10/PDF4–5,22: 2×2 repair; §7.1/F.2: MSE/decision inversion.</t>
+          <t>Chỉ ý tưởng; validation là kế hoạch (§3 tr2).</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>True-future diagnostic oracles có unequal info budgets; chưa chạy experiments.</t>
+          <t>Không số đo, không oracle/regret.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Center qua action pool không D20; E không D15 true oracle.</t>
+          <t>Không tách state/model; không định giá có kiểm soát.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/N/P</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Full bài</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>min2026misleads</t>
+          <t>dts25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Chỉ bối cảnh đoạn 1 related work.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -2300,42 +2600,42 @@
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AIS22</t>
+          <t>CEN26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
+          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Thông tin/model cần giữ gì để planning đủ tốt?</t>
+          <t>Telemetry model có cải thiện quyết định scheduling/provisioning không?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>History compression + reward/transition approximation.</t>
+          <t>Replay backfilling (5 walltime source, true runtime làm reference) và provisioning (§IV-A, §IV-D).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Def3/7,Thm5/9/PDF6–8,15–18: policy loss≤2αt.</t>
+          <t>CESNET vi phạm 20,5%→9,0% (§IV-D tr8); câu 'error saturates near last-value' trích từ [6] (§I).</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Uniform reward/IPM bounds; không full83pages hoặc chạy code.</t>
+          <t>Comparator hindsight; không oracle D15.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Không independent D20×D21 hoặc GM/Cref; chưa chứng nhận bound cho plant.</t>
+          <t>Không can thiệp state × model.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>P/N/N</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2345,22 +2645,18 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>subramanian2022ais</t>
+          <t>cen26</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Bối cảnh K-M1/K-M2.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2377,37 +2673,37 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>CEH23</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
+          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Điều kiện đủ để re-solving không làm hại?</t>
+          <t>Heuristic CE (thay bất định bằng giá trị danh nghĩa) cách tối ưu bao xa?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Sequential consistency + policy-objective accuracy.</t>
+          <t>CEC relaxation, update/projection/hybrid policy (§5); state hiện tại đầy đủ, W(t) quan sát trước quyết định (§2).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>§3 Def2–5/Props1–3/PDF8–10: SC+Π-accuracy⇒SI⇒non-deterioration.</t>
+          <t>Định lý 1–2 §6.1 tr21–22: C₁=O(√var), C₂=O(var); §8: re-solving không luôn có lợi (trích R02/R04).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>α bounds thường cần policy evaluation; chưa là usable predictive H1.</t>
+          <t>Assumption 5 động học affine; reward C³ lõm; queue phản xạ vi phạm.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>MP-feasibility khác action-feasibility; plant mapping là sufficient diagnostic.</t>
+          <t>Gần G_M|S1 nhưng không cho vị trí ranh giới trong plant phi tuyến.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -2422,22 +2718,18 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>secomandi2008resolving</t>
+          <t>ceh23</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Tác giả đọc §2 Assumption 5, §6.1 nếu dùng cho PC5; H1-Q04.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2454,37 +2746,37 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật allocation có thể hại?</t>
+          <t>NDT gate/utility regret trong networking đã có.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DLP re-solve theo capacity/conditional demand.</t>
+          <t>EWMA on-policy error + live-validated fallback.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§5 Example1/Eq10/PDF7: conditional revenue8.96→7.59; own full-expectation replay14.586589→14.079588.</t>
+          <t>§III–VI/PDF5–9: utility regret, feedback gate, injected neighbor-power offset.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Không rounding; không full asymptotic proofs/Phase3 hoặc RM four-cell replication.</t>
+          <t>Chưa chạy MATLAB; threshold chọn trên evaluation runs.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Multi-step booking khác one-shot queue; CE không cùng Jensen mechanism.</t>
+          <t>Không D20×D21; 21 power blends, khác one-shot queue.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -2499,7 +2791,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>R02 Example1 analytic replay</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2509,7 +2801,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>cooper2002asymptotic</t>
+          <t>almohammedi2026twinfidelity</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -2531,37 +2823,37 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Re-solving stochastic programming models for airline revenue management</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Vì sao SLP allocation re-solve không hại?</t>
+          <t>Sửa phần lỗi lớn nhất có cho action tốt nhất?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Integer allocation; objective bằng true policy expected revenue.</t>
+          <t>Matched-candidate center/response P,C,S,E grid.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TR Prop1/PDF10–11; §4/PDF16 bid-price có thể hại dù từ SLP.</t>
+          <t>§4–5/F.1 Eq10/PDF4–5,22: 2×2 repair; §7.1/F.2: MSE/decision inversion.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Journal proposition numbering chưa kiểm; không mọi policy/true MDP.</t>
+          <t>True-future diagnostic oracles có unequal info budgets; chưa chạy experiments.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Cùng proof structure K-S8, khác literal EVPPI và D20 intervention.</t>
+          <t>Center qua action pool không D20; E không D15 true oracle.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -2586,7 +2878,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>chen2010resolving</t>
+          <t>min2026misleads</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -2608,37 +2900,37 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
+          <t>Thông tin/model cần giữ gì để planning đủ tốt?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
+          <t>History compression + reward/transition approximation.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
+          <t>Def3/7,Thm5/9/PDF6–8,15–18: policy loss≤2αt.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
+          <t>Uniform reward/IPM bounds; không full83pages hoặc chạy code.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
+          <t>Không independent D20×D21 hoặc GM/Cref; chưa chứng nhận bound cho plant.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -2653,22 +2945,22 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm/chạy paper code</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>grimm2020valueequivalence</t>
+          <t>subramanian2022ais</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2685,37 +2977,37 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
+          <t>Điều kiện đủ để re-solving không làm hại?</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
+          <t>Sequential consistency + policy-objective accuracy.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
+          <t>§3 Def2–5/Props1–3/PDF8–10: SC+Π-accuracy⇒SI⇒non-deterioration.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
+          <t>α bounds thường cần policy evaluation; chưa là usable predictive H1.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
+          <t>MP-feasibility khác action-feasibility; plant mapping là sufficient diagnostic.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -2730,22 +3022,22 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Có link §2/PDF2; chưa chạy</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>1 (S2, 2026-10-24)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>amad2026dt2</t>
+          <t>secomandi2008resolving</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2762,37 +3054,37 @@
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Tối ưu TE khi future demand khó dự đoán.</t>
+          <t>Cập nhật allocation có thể hại?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
+          <t>DLP re-solve theo capacity/conditional demand.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
+          <t>§5 Example1/Eq10/PDF7: conditional revenue8.96→7.59; own full-expectation replay14.586589→14.079588.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
+          <t>Không rounding; không full asymptotic proofs/Phase3 hoặc RM four-cell replication.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
+          <t>Multi-step booking khác one-shot queue; CE không cùng Jensen mechanism.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -2807,22 +3099,22 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Có link §4.1; chưa chạy</t>
+          <t>R02 Example1 analytic replay</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>perry2023dote</t>
+          <t>cooper2002asymptotic</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -2839,37 +3131,37 @@
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
+          <t>Vì sao SLP allocation re-solve không hại?</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Aimsun + MPC structure-free 4 nút; I reference biết demand ghi sẵn → II aggregation → III bias trên aggregation (§2.1, §2.2.4).</t>
+          <t>Integer allocation; objective bằng true policy expected revenue.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Bias 1 đại lượng/lần (§3.3.1 tr15); Bảng 2 tr16 quét prediction 12/30/60 s và update 12/30/60 s; update ngắn bù một phần, state bias lớn làm mất bù (§3.3.2, §4).</t>
+          <t>TR Prop1/PDF10–11; §4/PDF16 bid-price có thể hại dù từ SLP.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Không joint bias (§4 tr18); solver heuristic &lt;1% so full B&amp;B (Fig3d); metric delay/xe so reference, không regret/oracle D15. Hình chỉ đọc caption.</t>
+          <t>Journal proposition numbering chưa kiểm; không mọi policy/true MDP.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
+          <t>Cùng proof structure K-S8, khác literal EVPPI và D20 intervention.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2884,22 +3176,22 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>4 (Crossref,2026-10-26)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>poelman2023structurefree</t>
+          <t>chen2010resolving</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2.4, §3.3, Bảng 2 nếu dùng cho nhãn PC2 ở L2.9; MT2/6/7 cập nhật ở follow-up.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -2916,42 +3208,42 @@
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
+          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
+          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
+          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
+          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
+          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>N/P/N</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2961,22 +3253,22 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Chưa kiểm/chạy paper code</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>mathijsen2017transient</t>
+          <t>grimm2020valueequivalence</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
+          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -2993,42 +3285,42 @@
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -3038,22 +3330,22 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Có link §2/PDF2; chưa chạy</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>amad2026dt2</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -3070,42 +3362,42 @@
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Tối ưu TE khi future demand khó dự đoán.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -3115,22 +3407,22 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Có link §4.1; chưa chạy</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>perry2023dote</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -3147,42 +3439,42 @@
     <row r="15" ht="84" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Aimsun + MPC structure-free 4 nút; I reference biết demand ghi sẵn → II aggregation → III bias trên aggregation (§2.1, §2.2.4).</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>Bias 1 đại lượng/lần (§3.3.1 tr15); Bảng 2 tr16 quét prediction 12/30/60 s và update 12/30/60 s; update ngắn bù một phần, state bias lớn làm mất bù (§3.3.2, §4).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>Không joint bias (§4 tr18); solver heuristic &lt;1% so full B&amp;B (Fig3d); metric delay/xe so reference, không regret/oracle D15. Hình chỉ đọc caption.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -3197,17 +3489,17 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>4 (Crossref,2026-10-26)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>poelman2023structurefree</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc §2.2.4, §3.3, Bảng 2 nếu dùng cho nhãn PC2 ở L2.9; MT2/6/7 cập nhật ở follow-up.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -3224,42 +3516,42 @@
     <row r="16" ht="84" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -3269,22 +3561,22 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>1 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -3294,49 +3586,49 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="17" ht="84" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -3346,22 +3638,22 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -3371,49 +3663,49 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -3423,18 +3715,22 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="n"/>
+          <t>Chưa kiểm code nguồn paper</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>128 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -3444,49 +3740,49 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="19" ht="84" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -3501,17 +3797,17 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>75 (S2, 2026-10-24)</t>
+          <t>117 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -3521,94 +3817,398 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="20" ht="84" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>NDT1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>185 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>almasan2022ndt</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="84" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>polverini2026conflicts</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>zhang2026opentwin</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="84" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Chưa đánh giá.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>P/P/P</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Metadata</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>34 (Crossref, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>kuri1995optimal</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Part 2b (L2.6).</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O20"/>
+  <autoFilter ref="A1:O24"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3623,7 +4223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -3650,228 +4250,240 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>19 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>23 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>L2.8 follow-up</t>
+          <t>Đợt duyệt 26/10</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>26/10: P02 nay có VoR do bạn tải; AI-T §1–5 + Bảng 2: bias một đại lượng mỗi lần, quét 1-D theo prediction/update horizon, không joint bias. Phiên tìm bổ sung lưu raw response; 3 đề xuất mới và 6 đề xuất cũ đã sàng abstract, chờ duyệt, chưa thêm hàng. Không L2.9/Gate.</t>
+          <t>Bạn duyệt và tải: IA26, DTS25, CEN26, CEH23 thêm vào đầu bảng (23 nguồn). Mức đọc ở Ghi_chu_doc là mức đọc thay bạn (AI-T/AI-F); cột Mức tôi đã đọc vẫn để bạn tự chọn. R06, 2211.01961, 2605.24318, 2505.04879, 2601.23051 lưu PDF nhưng không thêm hàng.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2</t>
+          <t>L2.8 follow-up</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
+          <t>26/10: P02 nay có VoR do bạn tải; AI-T §1–5 + Bảng 2: bias một đại lượng mỗi lần, quét 1-D theo prediction/update horizon, không joint bias. Phiên tìm bổ sung lưu raw response; 3 đề xuất mới và 6 đề xuất cũ đã sàng abstract, chờ duyệt, chưa thêm hàng. Không L2.9/Gate.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part B</t>
+          <t>L2.8 Part2</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
+          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part A</t>
+          <t>L2.7 Part B</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
+          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="38" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B20"/>
+  <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Check S11/R01/R34 versions, add T03 worked example and author reading pack
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có TR2006 (local); bản eCommons tác giả tải 26/10 = cùng TR; journal Annals OR chưa có</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>TR2006 AI-T; số mục bản journal 2010 **chưa kiểm** (cần bản Springer).</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>Có (arxivv3 local,42trang)</t>
+          <t>Có (journal TIT 72(4) 40 trang + arXiv v3)</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A: K3, controlled-source feedback, sampling-rate threshold.</t>
+          <t>Journal TIT2026 đã có; số mục §III/Eq10, §VII-D/Theorem9/Cor2/AppendixO khớp arXiv v3 (AI kiểm 26/10); chưa L-self.</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Paywall – cần thư viện</t>
+          <t>TAC 1995 chưa có; có bản CDC 1992 (2 trang) tác giả tải 26/10</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Queue / thông tin trễ: nguồn gần trục state; mới kiểm metadata, chưa đánh giá nội dung.</t>
+          <t>Bản CDC 1992 đọc 2 trang: JSEQ tối ưu khi trễ k=1, không tối ưu khi k≥2; cần TAC 1995 để kiểm chứng/phản ví dụ.</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>ia26</t>
@@ -2575,7 +2575,7 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>dts25</t>
@@ -2648,7 +2648,7 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>cen26</t>
@@ -2721,7 +2721,7 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
           <t>ceh23</t>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Cần bản journal Annals OR 177:91–114 để đối chiếu Prop1/Example3.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III/§VII-D; A4 kiểm freshness×model mismatch; P13 để Part B.</t>
+          <t>Tác giả đọc §III tr5–6 (Problem1 Eq10) bản journal.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -4148,12 +4148,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>CDC 1992 tr997–998: Thm2.1.2 JSEQ tối ưu với k=1; k≥2 có phản ví dụ (trỏ [4]); admission một queue: hai ngưỡng (Thm3.1.2).</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Chưa đọc.</t>
+          <t>Chỉ bản hội nghị 2 trang, chứng minh lược; mô hình đúng (không trục model).</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6).</t>
+          <t>Cần bản TAC 40(8) 1995.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gate L: GO có điều kiện with author-attested reading, T03 and label confirmation (DL-043)
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -995,7 +995,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -4223,7 +4223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4257,233 +4257,245 @@
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Đợt duyệt 26/10</t>
+          <t>Gate L 26/10</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Bạn duyệt và tải: IA26, DTS25, CEN26, CEH23 thêm vào đầu bảng (23 nguồn). Mức đọc ở Ghi_chu_doc là mức đọc thay bạn (AI-T/AI-F); cột Mức tôi đã đọc vẫn để bạn tự chọn. R06, 2211.01961, 2605.24318, 2505.04879, 2601.23051 lưu PDF nhưng không thêm hàng.</t>
+          <t>Bạn xác nhận (author-attested, DL-043) đã tự đọc WM26, R02, R04, P02, S11, P12 ở các mục ghi trong notes/literature/author_reading_record.md → Mức tôi đã đọc = Mục liên quan. P11 (archive) và T03 cũng attested. Các nguồn khác vẫn Chưa có xác nhận.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>L2.8 follow-up</t>
+          <t>Đợt duyệt 26/10</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>26/10: P02 nay có VoR do bạn tải; AI-T §1–5 + Bảng 2: bias một đại lượng mỗi lần, quét 1-D theo prediction/update horizon, không joint bias. Phiên tìm bổ sung lưu raw response; 3 đề xuất mới và 6 đề xuất cũ đã sàng abstract, chờ duyệt, chưa thêm hàng. Không L2.9/Gate.</t>
+          <t>Bạn duyệt và tải: IA26, DTS25, CEN26, CEH23 thêm vào đầu bảng (23 nguồn). Mức đọc ở Ghi_chu_doc là mức đọc thay bạn (AI-T/AI-F); cột Mức tôi đã đọc vẫn để bạn tự chọn. R06, 2211.01961, 2605.24318, 2505.04879, 2601.23051 lưu PDF nhưng không thêm hàng.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2</t>
+          <t>L2.8 follow-up</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
+          <t>26/10: P02 nay có VoR do bạn tải; AI-T §1–5 + Bảng 2: bias một đại lượng mỗi lần, quét 1-D theo prediction/update horizon, không joint bias. Phiên tìm bổ sung lưu raw response; 3 đề xuất mới và 6 đề xuất cũ đã sàng abstract, chờ duyệt, chưa thêm hàng. Không L2.9/Gate.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part B</t>
+          <t>L2.8 Part2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
+          <t>NDT26/WM26/AIS22 được duyệt; R04/R02/R01 được chỉ định. Cả6 AI-T, không L-self. WM26 có2×2repair; R04 sufficient diagnostic chưa khóa H1. A1–A3 bounded queries có checkpoint log nhưng thiếu raw từng rank; L2.9/Gate còn mở.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>L2.7 Part A</t>
+          <t>L2.7 Part B</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
+          <t>P12: VE Definition1/§3.1 AI-T. OεRE trong terms.md, không đổi contract; K5 chưa chọn. R43 chỉ tra bổ sung: abstract lượt này, old AI-T note có provenance. PartA còn P02 full text BLOCKED.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B</t>
+          <t>L2.7 Part A</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
+          <t>R51=P03 → P07 → P02: fidelity, oracle và factorial. P03/P07 AI-T; P02 chỉ abstract, full text BLOCKED. PartB/P12 đã có artifact riêng. Không tự cấp L-self/Gate.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part A</t>
+          <t>L2.6 Part B</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
+          <t>P13 → S11: backlog/horizon và freshness → decision cost. Hai parts đã thực hiện kỹ thuật; tác giả L-self/Gate/A4/L2.9 còn mở. T-H1 chỉ giới hạn diễn giải, không đổi metric.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2</t>
+          <t>L2.6 Part A</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
+          <t>S11: bản đọc arxivv3, journal identity TIT2026 đã kiểm. K3 ở notes/literature/freshness_decision_value.md; ghi chú PartA cũ là lịch sử.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1</t>
+          <t>L2.5 Part2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
+          <t>M00 → P04: herding theo tin cũ và fixed-M0 bias. Part2 đã kiểm kỹ thuật; tác giả L-self/Gate còn mở. P01 chỉ targeted screen, chưa cần đọc full.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>L2.4</t>
+          <t>L2.5 Part1</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
+          <t>P04: stale link-state, blocking và cost levels; Fig8 không phải clean2×2. Mức tác giả đọc cập nhật riêng, không tự nâng theo AI.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R32 / R34</t>
+          <t>L2.4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
+          <t>Nguồn lesson trước: NDT1 → P05 → P10. NMRG, P08, S07 tra bổ sung trong notes/literature/ndt_landscape.md.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>R51 = P03</t>
+          <t>R32 / R34</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
+          <t>Nguồn gần trục state: feedback control và queue với thông tin trễ; khác bài toán routing của repo.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Mức đọc</t>
+          <t>R51 = P03</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
+          <t>Một công trình DT², một hàng R51. Đã nâng AI note từ thứ cấp sang targeted PMLR; bản cũ có backup. DOTE/P07 là networking; P02 là nguồn phương pháp được chỉ định.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Mức đọc</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
+          <t>Bạn cập nhật Danh_sach → Mức tôi đã đọc; mức AI riêng ở Ghi_chu_doc. Giữ nguyên record cũ, không tự tăng mức đọc.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Tìm paper</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
+          <t>Ghi_chu_doc giữ nội dung theo ID; các nhắc lịch lesson trong ghi chú cũ là lịch sử. Mức AI đọc luôn tách khỏi mức bạn đọc.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lưu tạm</t>
+          <t>Tìm paper</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
+          <t>Dùng notes/literature/search_protocol.md; tác giả duyệt trước khi tải hoặc tạo note mới.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Nguồn lý thuyết</t>
+          <t>Lưu tạm</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
+          <t>archive/paper_comparison_part_a.xlsx giữ nguyên 21 bài và toàn bộ ghi chú trước dọn. Không phải yêu cầu đọc hết.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="38" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Link</t>
+          <t>Nguồn lý thuyết</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+          <t>SOB14, B82, P11 chỉ tra tên khái niệm khi cần; note/proof Part A vẫn ở notes/literature/.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="38" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Bấm DOI / Link hoặc PDF / Truy cập. Tên bài không gắn link; PDF chỉ mở trên máy có thư viện local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>E/M/R / ưu tiên</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Ước lượng AI từ lượt cũ; không tự chứng nhận novelty hay đổi nhãn PC/Gate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
L3R.4: freeze sourced worksheet and incomplete realism envelope before 216 labels
</commit_message>
<xml_diff>
--- a/papers/paper_comparison.xlsx
+++ b/papers/paper_comparison.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh_sach'!$A$1:$O$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Danh_sach'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ghi_chu_doc'!$A$1:$O$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Ghi_chu_doc'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Huong_dan'!$A$1:$B$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Huong_dan'!$1:$1</definedName>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,55 +567,55 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IA26</t>
+          <t>BAM10</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
+          <t>Network Traffic Characteristics of Data Centers in the Wild</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Scott Moeller; Bhaskar Krishnamachari</t>
+          <t>Theophilus Benson; Aditya Akella; David A. Maltz</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2026</v>
+        <v>2010</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>arXiv2609.06351v1</t>
+          <t>ACM IMC2010,267–280</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Theory / networked decisions</t>
+          <t>Data-center traffic measurement</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác nhận</t>
+          <t>Peer-reviewed publication identity checked; publisher direct access limited</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Networking/control: freshness × scope</t>
+          <t>Realism / networking</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>L3R.4</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC6: giá trị thông tin hiện tại theo decision-relevant predictability; môi trường ngoại sinh.</t>
+          <t>Q3R.3 / K9 / SR5–SR6; no PC relabel</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -630,67 +630,67 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2609.06351v1</t>
+          <t>doi:10.1145/1879141.1879175</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Đợt duyệt 26/10: AI-T §1–2.3, §3.4; chưa L-self.</t>
+          <t>L3R.4 targeted evidence, approved29/10; not author L-self</t>
         </is>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DTS25</t>
+          <t>ZLK17</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
+          <t>High-Resolution Measurement of Data Center Microbursts</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Zhiheng Yang; Francisco Vogt; Adam Belloum; Christian Rothenberg; Paola Grosso; Chrysa Papagianni</t>
+          <t>Qiao Zhang; Vincent Liu; Hongyi Zeng; Arvind Krishnamurthy</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2025</v>
+        <v>2017</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>CoNEXT'25 Student Workshop</t>
+          <t>ACM IMC2017,78–85</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Workshop (2 trang)</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Vision / NDT sync</t>
+          <t>Data-center microburst measurement</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Workshop sinh viên</t>
+          <t>Peer-reviewed publication identity checked; publisher direct access limited</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>NDT/networking</t>
+          <t>Realism / networking</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>L3R.4</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC6 framing: chọn telemetry theo giá trị quyết định; chưa có thí nghiệm.</t>
+          <t>Q3R.3 / K9 / SR5–SR6; no PC relabel</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -705,67 +705,67 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1145/3769700.3771695</t>
+          <t>doi:10.1145/3131365.3131375</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Đợt duyệt 26/10: AI-F 2 trang; chưa L-self.</t>
+          <t>L3R.4 targeted evidence, approved29/10; not author L-self</t>
         </is>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CEN26</t>
+          <t>LTWW94</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
+          <t>On the Self-Similar Nature of Ethernet Traffic (extended version)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Zifan Zhang; Zhichao Hou; Tingxiang Ji; Yuchen Liu</t>
+          <t>Will E. Leland; Murad S. Taqqu; Walter Willinger; Daniel V. Wilson</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2026</v>
+        <v>1994</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>arXiv2608.01725v1</t>
+          <t>IEEE/ACM ToN2(1):1–15</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Telemetry model / decision replay</t>
+          <t>Ethernet traffic measurement</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác nhận</t>
+          <t>Peer-reviewed publication identity checked; publisher direct access limited</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Networking/systems telemetry</t>
+          <t>Realism / networking</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>L3R.4</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>• PC5: đánh giá model bằng quyết định replay; không 2×2.</t>
+          <t>Q3R.3 / K9 / SR5–SR6; no PC relabel</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -780,37 +780,37 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2608.01725v1</t>
+          <t>doi:10.1109/90.282603</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Đợt duyệt 26/10: AI-T §I, §III-D, §IV-A, §IV-D; chưa L-self.</t>
+          <t>L3R.4 targeted evidence, approved29/10; not author L-self</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CEH23</t>
+          <t>IA26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
+          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Chen Yan; Alexandre Reiffers-Masson</t>
+          <t>Scott Moeller; Bhaskar Krishnamachari</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>arXiv2308.13166v1; submitted to Operations Research</t>
+          <t>arXiv2609.06351v1</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Stochastic optimization / CE bounds</t>
+          <t>Theory / networked decisions</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>OR / certainty equivalence</t>
+          <t>Networking/control: freshness × scope</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>• PC5/PC3: cận khoảng cách CE–tối ưu ∝√var hoặc var; cần động học affine trong kỳ vọng.</t>
+          <t>• PC2/PC6: giá trị thông tin hiện tại theo decision-relevant predictability; môi trường ngoại sinh.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -855,52 +855,52 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2308.13166v1</t>
+          <t>https://arxiv.org/abs/2609.06351v1</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Đợt duyệt 26/10: AI-T §2, §5.1, §6.1–6.3, §8; chưa L-self.</t>
+          <t>Đợt duyệt 26/10: AI-T §1–2.3, §3.4; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NDT26</t>
+          <t>DTS25</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
+          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Akram Almohammedi; Mohammed Balfaqih; Sam Darshi; Rami Langar; Wael Jaafar</t>
+          <t>Zhiheng Yang; Francisco Vogt; Adam Belloum; Christian Rothenberg; Paola Grosso; Chrysa Papagianni</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>arXiv2607.22857v1; submitted TNSM</t>
+          <t>CoNEXT'25 Student Workshop</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Workshop (2 trang)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Vision / NDT sync</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác nhận</t>
+          <t>Workshop sinh viên</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
+          <t>• PC2/PC6 framing: chọn telemetry theo giá trị quyết định; chưa có thí nghiệm.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -925,34 +925,34 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2607.22857v1</t>
+          <t>doi:10.1145/3769700.3771695</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-F 2 trang; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>WM26</t>
+          <t>CEN26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
+          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Rui Min; Xianyao Li; Fang Xu; Eric Jing Du (metadata: Jing Du)</t>
+          <t>Zifan Zhang; Zhichao Hou; Tingxiang Ji; Yuchen Liu</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -960,17 +960,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>arXiv2610.05550v1</t>
+          <t>arXiv2608.01725v1</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Preprint under review</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Telemetry model / decision replay</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -980,92 +980,92 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>World model/repair diagnosis</t>
+          <t>Networking/systems telemetry</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 framing AI đề xuất, không đổi nhãn.</t>
+          <t>• PC5: đánh giá model bằng quyết định replay; không 2×2.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Chưa có xác nhận</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2610.05550v1</t>
+          <t>https://arxiv.org/abs/2608.01725v1</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 framing; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-T §I, §III-D, §IV-A, §IV-D; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AIS22</t>
+          <t>CEH23</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
+          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Jayakumar Subramanian; Amit Sinha; Raihan Seraj; Aditya Mahajan</t>
+          <t>Chen Yan; Alexandre Reiffers-Masson</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>JMLR23(12):1–83</t>
+          <t>arXiv2308.13166v1; submitted to Operations Research</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Nguồn được yêu cầu/duyệt targeted</t>
+          <t>Stochastic optimization / CE bounds</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Partial observations/model adequacy</t>
+          <t>OR / certainty equivalence</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Tra khi cần</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
+          <t>• PC5/PC3: cận khoảng cách CE–tối ưu ∝√var hoặc var; cần động học affine trong kỳ vọng.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1075,47 +1075,47 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Có (local; targeted)</t>
+          <t>Có (local)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>https://www.jmlr.org/papers/v23/20-1165.html</t>
+          <t>https://arxiv.org/abs/2308.13166v1</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>Đợt duyệt 26/10: AI-T §2, §5.1, §6.1–6.3, §8; chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nicola Secomandi</t>
+          <t>Akram Almohammedi; Mohammed Balfaqih; Sam Darshi; Rami Langar; Wael Jaafar</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2008</v>
+        <v>2026</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>MSOM10(3):468–483</t>
+          <t>arXiv2607.22857v1; submitted TNSM</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>RM/conditions</t>
+          <t>NDT/networking</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1140,12 +1140,12 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>PC3/PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Chưa có xác nhận</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1155,42 +1155,42 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1287/msom.1070.0184</t>
+          <t>https://arxiv.org/abs/2607.22857v1</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>William L. Cooper</t>
+          <t>Rui Min; Xianyao Li; Fang Xu; Eric Jing Du (metadata: Jing Du)</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2002</v>
+        <v>2026</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Operations Research50(4):720–727</t>
+          <t>arXiv2610.05550v1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Preprint under review</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1200,22 +1200,22 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Chưa xác nhận</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>RM/negative information value</t>
+          <t>World model/repair diagnosis</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Tra khi cần</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>PC3; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>PC3/PC4; Tier1 framing AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1230,42 +1230,42 @@
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1287/opre.50.4.720.2855</t>
+          <t>https://arxiv.org/abs/2610.05550v1</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
+          <t>L2.8 Part2: Tier1 framing; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Re-solving stochastic programming models for airline revenue management</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Lijian Chen; Tito Homem-de-Mello</t>
+          <t>Jayakumar Subramanian; Amit Sinha; Raihan Seraj; Aditya Mahajan</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2010</v>
+        <v>2022</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Annals OR177:91–114; online2009</t>
+          <t>JMLR23(12):1–83</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc TR2006</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Có (journal)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>RM/non-deterioration</t>
+          <t>Partial observations/model adequacy</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
+          <t>PC5; Tier2 AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1300,52 +1300,52 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Có TR2006 (local); bản eCommons tác giả tải 26/10 = cùng TR; journal Annals OR chưa có</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s10479-009-0603-7</t>
+          <t>https://www.jmlr.org/papers/v23/20-1165.html</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>TR2006 AI-T; số mục bản journal 2010 **chưa kiểm** (cần bản Springer).</t>
+          <t>L2.8 Part2: Tier2; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
+          <t>Nicola Secomandi</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2020</v>
+        <v>2008</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>NeurIPS33</t>
+          <t>MSOM10(3):468–483</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Khái niệm / model-based RL</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Value equivalence / decision-relevant models</t>
+          <t>RM/conditions</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1375,52 +1375,52 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Có (NeurIPS12trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
+          <t>doi:10.1287/msom.1070.0184</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Harry Amad; Mihaela van der Schaar</t>
+          <t>William L. Cooper</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2026</v>
+        <v>2002</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>ICML2026, PMLR306:2207–2233</t>
+          <t>Operations Research50(4):720–727</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1430,92 +1430,92 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>A1/A5 Decision-targeted twin</t>
+          <t>RM/negative information value</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
+          <t>PC3; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Có (PMLR27trang local)</t>
+          <t>Có (local; targeted)</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
+          <t>doi:10.1287/opre.50.4.720.2855</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
+          <t>L2.8 Part2: Tier1 priority; AI-T, chưa L-self. Không phải yêu cầu đọc full.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
+          <t>Lijian Chen; Tito Homem-de-Mello</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2023</v>
+        <v>2010</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>USENIX NSDI23:1557–1581</t>
+          <t>Annals OR177:91–114; online2009</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Conference (đọc proceedings)</t>
+          <t>Journal; đọc TR2006</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Phương pháp / empirical TE</t>
+          <t>Nguồn được yêu cầu/duyệt targeted</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>WAN traffic engineering / direct optimization</t>
+          <t>RM/non-deterioration</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Tra khi cần</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
+          <t>PC3/PC4; Tier1 priority AI đề xuất, không đổi nhãn.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1525,52 +1525,52 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Có (USENIX26trang gồm cover)</t>
+          <t>Có TR2006 (local); bản eCommons tác giả tải 26/10 = cùng TR; journal Annals OR chưa có</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
+          <t>doi:10.1007/s10479-009-0603-7</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
+          <t>TR2006 AI-T; số mục bản journal 2010 **chưa kiểm** (cần bản Springer).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="72" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
+          <t>Christopher Grimm; André Barreto; Satinder P. Singh; David Silver</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>TR-C153:104174</t>
+          <t>NeurIPS33</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Journal (VoR, CC BY)</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity / predictive control</t>
+          <t>Khái niệm / model-based RL</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1580,17 +1580,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Control methodology / nguồn tác giả chỉ định</t>
+          <t>Value equivalence / decision-relevant models</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>• PC2 (PHASE_2 v2.0 §5.4: nguồn quyết định nhãn) / PC3/PC4/PC5: bias một đại lượng mỗi lần; sweep 1-D theo prediction/update horizon; không gán dấu Γ.</t>
+          <t>• PC5/PC3: model sufficiency đã có; không phải clearance OεRE.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1600,52 +1600,52 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Có (VoR 20 trang local; tác giả tải 26/10)</t>
+          <t>Có (NeurIPS12trang local)</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1016/j.trc.2023.104174</t>
+          <t>https://proceedings.neurips.cc/paper/2020/hash/3bb585ea00014b0e3ebe4c6dd165a358-Abstract.html</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA dependency: AI-T VoR §1–5 + Bảng 2 (L2.8 follow-up 26/10); chưa L-self.</t>
+          <t>L2.7 PartB: Definition1/§3.1 AI-T, chưa L-self; R43/AVE là nguồn khác, tra bổ sung.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="72" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Britt Mathijsen; Bert Zwart</t>
+          <t>Harry Amad; Mihaela van der Schaar</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>2017</v>
+        <v>2026</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Queueing Systems85(3–4):269–304</t>
+          <t>ICML2026, PMLR306:2207–2233</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Journal (đọc VoR CWI)</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Lý thuyết / numerical study</t>
+          <t>Phương pháp</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Queueing / transient approximation / staffing</t>
+          <t>A1/A5 Decision-targeted twin</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
+          <t>• PC2/PC3/PC4/PC5: decision fidelity và regret đã có; không xác nhận D19Γ.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1675,62 +1675,62 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Có (journal36trang local)</t>
+          <t>Có (PMLR27trang local)</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1007/s11134-016-9511-0</t>
+          <t>https://proceedings.mlr.press/v306/amad26a.html</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
+          <t>L2.7 PartA hiện tại; R51=P03, cùng một bài. AI-T PMLR, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="72" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
+          <t>Yarin Perry; Felipe Vieira Frujeri; Chaim Hoch; Srikanth Kandula; Ishai Menache; Michael Schapira; Aviv Tamar</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>IEEE TIT72(4):2237–2276</t>
+          <t>USENIX NSDI23:1557–1581</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Journal; đọc arxivv3</t>
+          <t>Conference (đọc proceedings)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / tối ưu</t>
+          <t>Phương pháp / empirical TE</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Có (identity đã kiểm)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Networking / goal-oriented remote decisions</t>
+          <t>WAN traffic engineering / direct optimization</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1740,137 +1740,137 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
+          <t>• PC2/PC5: decision-aligned objective; PC3/PC4: oracle/design boundary.</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Chưa có xác nhận</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>Có (journal TIT 72(4) 40 trang + arXiv v3)</t>
+          <t>Có (USENIX26trang gồm cover)</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TIT.2026.3663678</t>
+          <t>https://www.usenix.org/conference/nsdi23/presentation/perry</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Journal TIT2026 đã có; số mục §III/Eq10, §VII-D/Theorem9/Cor2/AppendixO khớp arXiv v3 (AI kiểm 26/10); chưa L-self.</t>
+          <t>L2.7 PartA: networking prior, oracle biết future demands; AI-T, chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="72" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Michael Mitzenmacher</t>
+          <t>M. C. Poelman; A. Hegyi; A. Verbraeck; J. W. C. van Lint</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>2000</v>
+        <v>2023</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>IEEE TPDS11(1):6–20</t>
+          <t>TR-C153:104174</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Journal; PDF là submission</t>
+          <t>Journal (VoR, CC BY)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Mô hình / simulation</t>
+          <t>Sensitivity / predictive control</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Có (journal identity)</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Networking / load balancing, stale queues</t>
+          <t>Control methodology / nguồn tác giả chỉ định</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
+          <t>• PC2 (PHASE_2 v2.0 §5.4: nguồn quyết định nhãn) / PC3/PC4/PC5: bias một đại lượng mỗi lần; sweep 1-D theo prediction/update horizon; không gán dấu Γ.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>Có (submission28trang local)</t>
+          <t>Có (VoR 20 trang local; tác giả tải 26/10)</t>
         </is>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/71.824633</t>
+          <t>doi:10.1016/j.trc.2023.104174</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
+          <t>L2.7 PartA dependency: AI-T VoR §1–5 + Bảng 2 (L2.8 follow-up 26/10); chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="72" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Shaikh, Rexford, Shin</t>
+          <t>Britt Mathijsen; Bert Zwart</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2001</v>
+        <v>2017</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>IEEE/ACM ToN9(2):162–176</t>
+          <t>Queueing Systems85(3–4):269–304</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal (đọc VoR CWI)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Thực nghiệm / đánh giá</t>
+          <t>Lý thuyết / numerical study</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>QoS routing / stale link-state</t>
+          <t>Queueing / transient approximation / staffing</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
+          <t>• PC3/PC4/PC6: prior về horizon/initial workload; không transfer trực tiếp sang binary routing.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1900,62 +1900,62 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (journal36trang local)</t>
         </is>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/90.917073</t>
+          <t>doi:10.1007/s11134-016-9511-0</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
+          <t>L2.6 Part B: normalized vs cumulative cost, continuous vs binary, T-H1.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="72" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Almasan et al.</t>
+          <t>Aimin Li, Shaohua Wu, Gary C. F. Lee, Sumei Sun</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>IEEE Communications Magazine 60(11):22–27</t>
+          <t>IEEE TIT72(4):2237–2276</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Journal; đọc arxivv3</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Survey</t>
+          <t>Mô hình / tối ưu</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (identity đã kiểm)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>NDT / routing what-if</t>
+          <t>Networking / goal-oriented remote decisions</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1965,72 +1965,72 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+          <t>• PC2/PC3/PC4/PC6: decision-aware freshness đã có; không novelty clearance.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Chưa có xác nhận</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Có (local)</t>
+          <t>Có (journal TIT 72(4) 40 trang + arXiv v3)</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/MCOM.001.2200012</t>
+          <t>doi:10.1109/TIT.2026.3663678</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+          <t>Journal TIT2026 đã có; số mục §III/Eq10, §VII-D/Theorem9/Cor2/AppendixO khớp arXiv v3 (AI kiểm 26/10); chưa L-self.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="72" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Polverini et al.</t>
+          <t>Michael Mitzenmacher</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2026</v>
+        <v>2000</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>IEEE TNSM23:2038–2050</t>
+          <t>IEEE TPDS11(1):6–20</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Journal; PDF là submission</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Mô hình / simulation</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Có (journal identity)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>NDT / SDN conflict detection</t>
+          <t>Networking / load balancing, stale queues</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+          <t>• PC2/PC3/PC4/PC6: policy×delay, herding, baseline; không novelty clearance.</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2048,64 +2048,64 @@
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Full text web; PDF local403</t>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Có (submission28trang local)</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>doi:10.1109/TNSM.2026.3652800</t>
+          <t>doi:10.1109/71.824633</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+          <t>L2.5 Part2: herding khác V1 model bias; K-S3/K-S4.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="72" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+          <t>Shaikh, Rexford, Shin</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2026</v>
+        <v>2001</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>arXiv:2605.24662v2 (preprint)</t>
+          <t>IEEE/ACM ToN9(2):162–176</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Thực nghiệm / đánh giá</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Chưa rõ</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>O-RAN / online calibration / gate</t>
+          <t>QoS routing / stale link-state</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+          <t>• State cũ, routing đổi tải; prior cho wording PC2/PC3/PC4/PC6.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2130,29 +2130,29 @@
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2605.24662v2</t>
+          <t>doi:10.1109/90.917073</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+          <t>L2.5 Part1: đọc chính P04; kiểm §V-A/Fig8 trước dùng cho PC3.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Soleymani, Baras, Hirche</t>
+          <t>Almasan et al.</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -2160,140 +2160,365 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
+          <t>IEEE Communications Magazine 60(11):22–27</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Magazine</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>NDT / routing what-if</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>• Định vị giá trị thông tin và model trong quyết định routing.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/MCOM.001.2200012</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 1: vocabulary, pipeline và routing optimizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Polverini et al.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>IEEE TNSM23:2038–2050</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>NDT / SDN conflict detection</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>• Prior cho twin đánh giá action làm đổi tải; metric khác expected regret.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Full text web; PDF local403</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>doi:10.1109/TNSM.2026.3652800</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 2: passive feedback và verdict metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Zhang, Hossen, Ron, Shah, Liu</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24662v2 (preprint)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Chưa rõ</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>O-RAN / online calibration / gate</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>• Đối chiếu thông tin/model và chất lượng quyết định; không tự gán same intervention.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có xác nhận</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>Có (local)</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2605.24662v2</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>L2.4 đọc chính 3: calibrate/resync và gate trước action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Soleymani, Baras, Hirche</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>IEEE TAC 67(7)</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>A2 VoI trong control</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18
 • Sửa state lợi hơn sửa model ít nhất 1% ở các ô M09–M12</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>Có (local)</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/TAC.2021.3113472</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>State / networked control: đối chiếu giá trị thông tin; không tự suy ra tương tác state–model.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="72" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Kuri, Kumar</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D27" s="2" t="n">
         <v>1995</v>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>IEEE TAC 40(8)</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>A6 Queue, thông tin trễ</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>• Thấy mode có lợi hơn làm mới backlog ở các ô M17, M18</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>Chưa có xác nhận</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>TAC 1995 chưa có; có bản CDC 1992 (2 trang) tác giả tải 26/10</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="N27" s="3" t="inlineStr">
         <is>
           <t>doi:10.1109/9.402238</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>Bản CDC 1992 đọc 2 trang: JSEQ tối ưu khi trễ k=1, không tối ưu khi k≥2; cần TAC 1995 để kiểm chứng/phản ví dụ.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O24"/>
+  <autoFilter ref="A1:O27"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Chưa có xác nhận,Chưa đọc,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2336,12 +2561,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -2354,7 +2585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2454,42 +2685,42 @@
     <row r="2" ht="84" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IA26</t>
+          <t>BAM10</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
+          <t>Network Traffic Characteristics of Data Centers in the Wild</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Thông tin mới-cục bộ hay đầy đủ-trễ cho quyết định đội?</t>
+          <t>Do measurements supply comparable realism bounds?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Cost bậc hai, x*=Q⁻¹b(θ_t); regret so thông tin hiện tại đầy đủ (§2.3 Eq19–21).</t>
+          <t>Data-center traffic measurement</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Định lý 3 §3.4 tr13–14: fresh-local thắng ⇔ τ/T &gt; ½log(1/(1−η_S(0))); Eq22–23: thêm thông tin cùng độ tươi không hại.</t>
+          <t>Data center10sites; SNMP1–30min; ON/OFF theo arrival95; §3.1/PDF3,§5.2/PDF6–7/Table4,§6.2–6.3/PDF9</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Môi trường không bị action điều khiển; loại trừ controlled queueing (§1 tr3).</t>
+          <t>Heavy-tail structure; coarse utilization does not bound offered-rate peak</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Không trục model, không Γ; repo là quyết định làm đổi tải có mode ẩn.</t>
+          <t>Measurements of real network traffic, no repo decision estimand or contrast</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>P/N/N</t>
+          <t>N/N/N</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2499,18 +2730,18 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="n"/>
+          <t>Không lấy dữ liệu/code trong phiên này</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>ia26</t>
+          <t>bam10</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.3, §3.4 nếu dùng cho PC6.</t>
+          <t>Source matched backlog AoI / offered input / buffer-time / holding horizon</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -2520,70 +2751,70 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DTS25</t>
+          <t>ZLK17</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
+          <t>High-Resolution Measurement of Data Center Microbursts</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Đo gì, ở đâu, khi nào để đồng bộ NDT dưới ngân sách?</t>
+          <t>Do measurements supply comparable realism bounds?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Neural Measurement Field λθ(e,t,f,p|z_c) học online (§2).</t>
+          <t>Data-center microburst measurement</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chỉ ý tưởng; validation là kế hoạch (§3 tr2).</t>
+          <t>30racks; byte counters25µs; egress hot&gt;50%;p90burst&lt;200µs; §4/PDF3–4,§5/PDF4–5,§6.4/PDF7</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Không số đo, không oracle/regret.</t>
+          <t>Egress hot-duration != hidden holding time; normalized shared-buffer occupancy != absolute budget</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Không tách state/model; không định giá có kiểm soát.</t>
+          <t>Measurements of real network traffic, no repo decision estimand or contrast</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>N/N/P</t>
+          <t>N/N/N</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Full bài</t>
+          <t>Mục liên quan</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n"/>
+          <t>Không lấy dữ liệu/code trong phiên này</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>dts25</t>
+          <t>zlk17</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Chỉ bối cảnh đoạn 1 related work.</t>
+          <t>Source matched backlog AoI / offered input / buffer-time / holding horizon</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -2593,49 +2824,49 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CEN26</t>
+          <t>LTWW94</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
+          <t>On the Self-Similar Nature of Ethernet Traffic (extended version)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Telemetry model có cải thiện quyết định scheduling/provisioning không?</t>
+          <t>Do measurements supply comparable realism bounds?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Replay backfilling (5 walltime source, true runtime làm reference) và provisioning (§IV-A, §IV-D).</t>
+          <t>Ethernet traffic measurement</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>CESNET vi phạm 20,5%→9,0% (§IV-D tr8); câu 'error saturates near last-value' trích từ [6] (§I).</t>
+          <t>Bellcore1989–92; multiscale variability/IDC; journal extended version; PDF1–2/TableI,§3.1/PDF4,§4/PDF7–8,§5.2/PDF12</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Comparator hindsight; không oracle D15.</t>
+          <t>Historical LAN not modern edge envelope; IDC != window-rate CV</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Không can thiệp state × model.</t>
+          <t>Measurements of real network traffic, no repo decision estimand or contrast</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>P/N/N</t>
+          <t>N/N/N</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2645,18 +2876,18 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="n"/>
+          <t>Không lấy dữ liệu/code trong phiên này</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>cen26</t>
+          <t>ltww94</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh K-M1/K-M2.</t>
+          <t>Source matched backlog AoI / offered input / buffer-time / holding horizon</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2666,49 +2897,49 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CEH23</t>
+          <t>IA26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
+          <t>A Theory of Information Architecture for Networked Decisions: Freshness, Locality, and Coordination</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Heuristic CE (thay bất định bằng giá trị danh nghĩa) cách tối ưu bao xa?</t>
+          <t>Thông tin mới-cục bộ hay đầy đủ-trễ cho quyết định đội?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>CEC relaxation, update/projection/hybrid policy (§5); state hiện tại đầy đủ, W(t) quan sát trước quyết định (§2).</t>
+          <t>Cost bậc hai, x*=Q⁻¹b(θ_t); regret so thông tin hiện tại đầy đủ (§2.3 Eq19–21).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Định lý 1–2 §6.1 tr21–22: C₁=O(√var), C₂=O(var); §8: re-solving không luôn có lợi (trích R02/R04).</t>
+          <t>Định lý 3 §3.4 tr13–14: fresh-local thắng ⇔ τ/T &gt; ½log(1/(1−η_S(0))); Eq22–23: thêm thông tin cùng độ tươi không hại.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Assumption 5 động học affine; reward C³ lõm; queue phản xạ vi phạm.</t>
+          <t>Môi trường không bị action điều khiển; loại trừ controlled queueing (§1 tr3).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Gần G_M|S1 nhưng không cho vị trí ranh giới trong plant phi tuyến.</t>
+          <t>Không trục model, không Γ; repo là quyết định làm đổi tải có mode ẩn.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>P/N/N</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -2724,12 +2955,12 @@
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>ceh23</t>
+          <t>ia26</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2 Assumption 5, §6.1 nếu dùng cho PC5; H1-Q04.</t>
+          <t>Tác giả đọc §2.3, §3.4 nếu dùng cho PC6.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2746,67 +2977,63 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NDT26</t>
+          <t>DTS25</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
+          <t>Adaptive Digital Twin Synchronization: A Mechanism for Where, When, and What to Measure</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>NDT gate/utility regret trong networking đã có.</t>
+          <t>Đo gì, ở đâu, khi nào để đồng bộ NDT dưới ngân sách?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>EWMA on-policy error + live-validated fallback.</t>
+          <t>Neural Measurement Field λθ(e,t,f,p|z_c) học online (§2).</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>§III–VI/PDF5–9: utility regret, feedback gate, injected neighbor-power offset.</t>
+          <t>Chỉ ý tưởng; validation là kế hoạch (§3 tr2).</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy MATLAB; threshold chọn trên evaluation runs.</t>
+          <t>Không số đo, không oracle/regret.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Không D20×D21; 21 power blends, khác one-shot queue.</t>
+          <t>Không tách state/model; không định giá có kiểm soát.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/N/P</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Mục liên quan</t>
+          <t>Full bài</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>almohammedi2026twinfidelity</t>
+          <t>dts25</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Chỉ bối cảnh đoạn 1 related work.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -2823,42 +3050,42 @@
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>WM26</t>
+          <t>CEN26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
+          <t>CENTILE: A Telemetry Foundation Model Evaluated by the Decisions It Drives</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Sửa phần lỗi lớn nhất có cho action tốt nhất?</t>
+          <t>Telemetry model có cải thiện quyết định scheduling/provisioning không?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Matched-candidate center/response P,C,S,E grid.</t>
+          <t>Replay backfilling (5 walltime source, true runtime làm reference) và provisioning (§IV-A, §IV-D).</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>§4–5/F.1 Eq10/PDF4–5,22: 2×2 repair; §7.1/F.2: MSE/decision inversion.</t>
+          <t>CESNET vi phạm 20,5%→9,0% (§IV-D tr8); câu 'error saturates near last-value' trích từ [6] (§I).</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>True-future diagnostic oracles có unequal info budgets; chưa chạy experiments.</t>
+          <t>Comparator hindsight; không oracle D15.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Center qua action pool không D20; E không D15 true oracle.</t>
+          <t>Không can thiệp state × model.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>P/N/N</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -2868,22 +3095,18 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>min2026misleads</t>
+          <t>cen26</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Bối cảnh K-M1/K-M2.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2900,37 +3123,37 @@
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AIS22</t>
+          <t>CEH23</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
+          <t>Certainty Equivalence Control-Based Heuristics in Multi-Stage Convex Stochastic Optimization Problems</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Thông tin/model cần giữ gì để planning đủ tốt?</t>
+          <t>Heuristic CE (thay bất định bằng giá trị danh nghĩa) cách tối ưu bao xa?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>History compression + reward/transition approximation.</t>
+          <t>CEC relaxation, update/projection/hybrid policy (§5); state hiện tại đầy đủ, W(t) quan sát trước quyết định (§2).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Def3/7,Thm5/9/PDF6–8,15–18: policy loss≤2αt.</t>
+          <t>Định lý 1–2 §6.1 tr21–22: C₁=O(√var), C₂=O(var); §8: re-solving không luôn có lợi (trích R02/R04).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Uniform reward/IPM bounds; không full83pages hoặc chạy code.</t>
+          <t>Assumption 5 động học affine; reward C³ lõm; queue phản xạ vi phạm.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Không independent D20×D21 hoặc GM/Cref; chưa chứng nhận bound cho plant.</t>
+          <t>Gần G_M|S1 nhưng không cho vị trí ranh giới trong plant phi tuyến.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -2945,22 +3168,18 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy paper code</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Chưa kiểm citation count lượt này</t>
-        </is>
-      </c>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>subramanian2022ais</t>
+          <t>ceh23</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
+          <t>Tác giả đọc §2 Assumption 5, §6.1 nếu dùng cho PC5; H1-Q04.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2977,37 +3196,37 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>R04</t>
+          <t>NDT26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
+          <t>Twin-Fidelity-Aware Resolution of Direct xApp Conflicts in Open RAN</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Điều kiện đủ để re-solving không làm hại?</t>
+          <t>NDT gate/utility regret trong networking đã có.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Sequential consistency + policy-objective accuracy.</t>
+          <t>EWMA on-policy error + live-validated fallback.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>§3 Def2–5/Props1–3/PDF8–10: SC+Π-accuracy⇒SI⇒non-deterioration.</t>
+          <t>§III–VI/PDF5–9: utility regret, feedback gate, injected neighbor-power offset.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>α bounds thường cần policy evaluation; chưa là usable predictive H1.</t>
+          <t>Chưa chạy MATLAB; threshold chọn trên evaluation runs.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>MP-feasibility khác action-feasibility; plant mapping là sufficient diagnostic.</t>
+          <t>Không D20×D21; 21 power blends, khác one-shot queue.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -3032,7 +3251,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>secomandi2008resolving</t>
+          <t>almohammedi2026twinfidelity</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -3054,37 +3273,37 @@
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>R02</t>
+          <t>WM26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
+          <t>When Low Prediction Error Misleads Planning: Diagnosing Representation, Dynamics, and Decision Failures in Latent World Models</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật allocation có thể hại?</t>
+          <t>Sửa phần lỗi lớn nhất có cho action tốt nhất?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>DLP re-solve theo capacity/conditional demand.</t>
+          <t>Matched-candidate center/response P,C,S,E grid.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>§5 Example1/Eq10/PDF7: conditional revenue8.96→7.59; own full-expectation replay14.586589→14.079588.</t>
+          <t>§4–5/F.1 Eq10/PDF4–5,22: 2×2 repair; §7.1/F.2: MSE/decision inversion.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Không rounding; không full asymptotic proofs/Phase3 hoặc RM four-cell replication.</t>
+          <t>True-future diagnostic oracles có unequal info budgets; chưa chạy experiments.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Multi-step booking khác one-shot queue; CE không cùng Jensen mechanism.</t>
+          <t>Center qua action pool không D20; E không D15 true oracle.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -3099,7 +3318,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>R02 Example1 analytic replay</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3109,7 +3328,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>cooper2002asymptotic</t>
+          <t>min2026misleads</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -3131,37 +3350,37 @@
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>R01</t>
+          <t>AIS22</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Re-solving stochastic programming models for airline revenue management</t>
+          <t>Approximate Information State for Approximate Planning and Reinforcement Learning in Partially Observed Systems</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Vì sao SLP allocation re-solve không hại?</t>
+          <t>Thông tin/model cần giữ gì để planning đủ tốt?</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Integer allocation; objective bằng true policy expected revenue.</t>
+          <t>History compression + reward/transition approximation.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TR Prop1/PDF10–11; §4/PDF16 bid-price có thể hại dù từ SLP.</t>
+          <t>Def3/7,Thm5/9/PDF6–8,15–18: policy loss≤2αt.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Journal proposition numbering chưa kiểm; không mọi policy/true MDP.</t>
+          <t>Uniform reward/IPM bounds; không full83pages hoặc chạy code.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Cùng proof structure K-S8, khác literal EVPPI và D20 intervention.</t>
+          <t>Không independent D20×D21 hoặc GM/Cref; chưa chứng nhận bound cho plant.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -3186,12 +3405,12 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>chen2010resolving</t>
+          <t>subramanian2022ais</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Cần bản journal Annals OR 177:91–114 để đối chiếu Prop1/Example3.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -3208,37 +3427,37 @@
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>R04</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
+          <t>An Analysis of the Control-Algorithm Re-solving Issue in Inventory and Revenue Management</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
+          <t>Điều kiện đủ để re-solving không làm hại?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
+          <t>Sequential consistency + policy-objective accuracy.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
+          <t>§3 Def2–5/Props1–3/PDF8–10: SC+Π-accuracy⇒SI⇒non-deterioration.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
+          <t>α bounds thường cần policy evaluation; chưa là usable predictive H1.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
+          <t>MP-feasibility khác action-feasibility; plant mapping là sufficient diagnostic.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -3253,22 +3472,22 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm/chạy paper code</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>grimm2020valueequivalence</t>
+          <t>secomandi2008resolving</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -3285,37 +3504,37 @@
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>R51</t>
+          <t>R02</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>DT²: Decision-Targeted Digital Twins</t>
+          <t>Asymptotic Behavior of an Allocation Policy for Revenue Management</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
+          <t>Cập nhật allocation có thể hại?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
+          <t>DLP re-solve theo capacity/conditional demand.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
+          <t>§5 Example1/Eq10/PDF7: conditional revenue8.96→7.59; own full-expectation replay14.586589→14.079588.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
+          <t>Không rounding; không full asymptotic proofs/Phase3 hoặc RM four-cell replication.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
+          <t>Multi-step booking khác one-shot queue; CE không cùng Jensen mechanism.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -3330,22 +3549,22 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Có link §2/PDF2; chưa chạy</t>
+          <t>R02 Example1 analytic replay</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>1 (S2, 2026-10-24)</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>amad2026dt2</t>
+          <t>cooper2002asymptotic</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
+          <t>Tác giả đọc đúng câu hỏi trong note; L2.9 chấm prior boundary, không tự mở Phase3.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -3362,37 +3581,37 @@
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>R01</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
+          <t>Re-solving stochastic programming models for airline revenue management</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Tối ưu TE khi future demand khó dự đoán.</t>
+          <t>Vì sao SLP allocation re-solve không hại?</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
+          <t>Integer allocation; objective bằng true policy expected revenue.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
+          <t>TR Prop1/PDF10–11; §4/PDF16 bid-price có thể hại dù từ SLP.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
+          <t>Journal proposition numbering chưa kiểm; không mọi policy/true MDP.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
+          <t>Cùng proof structure K-S8, khác literal EVPPI và D20 intervention.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -3407,22 +3626,22 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Có link §4.1; chưa chạy</t>
+          <t>Chưa chạy paper code</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm lượt này</t>
+          <t>Chưa kiểm citation count lượt này</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>perry2023dote</t>
+          <t>chen2010resolving</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
+          <t>Cần bản journal Annals OR 177:91–114 để đối chiếu Prop1/Example3.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -3439,37 +3658,37 @@
     <row r="15" ht="84" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
+          <t>The Value Equivalence Principle for Model-Based Reinforcement Learning</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
+          <t>Model cần giữ thông tin gì để phục vụ value-based planning?</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Aimsun + MPC structure-free 4 nút; I reference biết demand ghi sẵn → II aggregation → III bias trên aggregation (§2.1, §2.2.4).</t>
+          <t>VE: equal Bellman updates cho Π,V; class co lại khi test sets lớn hơn.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Bias 1 đại lượng/lần (§3.3.1 tr15); Bảng 2 tr16 quét prediction 12/30/60 s và update 12/30/60 s; update ngắn bù một phần, state bias lớn làm mất bù (§3.3.2, §4).</t>
+          <t>§3 Def1/PDF3; §3.1 Properties1–4/PDF3–4. Exact operator equality, không trực tiếp OεRE.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Không joint bias (§4 tr18); solver heuristic &lt;1% so full B&amp;B (Fig3d); metric delay/xe so reference, không regret/oracle D15. Hình chỉ đọc caption.</t>
+          <t>Targeted definition/properties; proofs/experiments chưa đọc. R43 current abstract, old AI-T provenance riêng.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
+          <t>OεRE đo true policy cost difference theo pipeline/ô; VE chỉ thành exact J fidelity dưới macro one-step embedding.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -3484,22 +3703,22 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm/chạy paper code</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>4 (Crossref,2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>poelman2023structurefree</t>
+          <t>grimm2020valueequivalence</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §2.2.4, §3.3, Bảng 2 nếu dùng cho nhãn PC2 ở L2.9; MT2/6/7 cập nhật ở follow-up.</t>
+          <t>Tác giả đọc Def1/§3.1; A3/A4 kiểm AVE quantifiers; không nhận OεRE là mới.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -3516,42 +3735,42 @@
     <row r="16" ht="84" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>R51</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Transient error approximation in a Lévy queue</t>
+          <t>DT²: Decision-Targeted Digital Twins</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
+          <t>Simulation fidelity tốt có bảo đảm chọn đúng policy?</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
+          <t>Ranking loss + FQE cho learned DT; không phải D21.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
+          <t>§3 Thm3.1: tồn tại reward/Π xếp sai dưới KL assumptions; §6.2: expected regret, MC500rollouts/policy (B.4.2).</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
+          <t>Thm tồn tại, không tần suất; finite policy set; FQE coverage, §7.1; AI-T chọn lọc.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
+          <t>Repo dùng M0/M1 cố định, one-shot và controlled state×model.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>N/P/N</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -3561,22 +3780,22 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Có link §2/PDF2; chưa chạy</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-26)</t>
+          <t>1 (S2, 2026-10-24)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>mathijsen2017transient</t>
+          <t>amad2026dt2</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
+          <t>L2.7 PartA: tác giả đọc targeted; A4/L2.8/L2.9/Gate còn mở.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -3593,42 +3812,42 @@
     <row r="17" ht="84" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
+          <t>DOTE: Rethinking (Predictive) WAN Traffic Engineering</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
+          <t>Tối ưu TE khi future demand khó dự đoán.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
+          <t>Historical demand → split ratios, tối ưu thẳng TE objective (§2.2–3.2).</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
+          <t>§4.1/tr1564–1565: ratio so oracle biết future demands; không cùng D15/regret.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
+          <t>§3.3 idealized expressive mapping/stationary sampling; không guarantee DNN thực đạt global optimum.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
+          <t>Repeated TE/trace + hindsight ratio; repo one-shot expected-cost oracle.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -3638,22 +3857,22 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Chưa chạy code paper</t>
+          <t>Có link §4.1; chưa chạy</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>6 (Crossref, 2026-10-26)</t>
+          <t>Chưa kiểm lượt này</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>li2026freshness</t>
+          <t>perry2023dote</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III tr5–6 (Problem1 Eq10) bản journal.</t>
+          <t>Tác giả đọc §2.2/3.1–3.3/4.1; giữ riêng mức AI/tác giả.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -3670,42 +3889,42 @@
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>M00</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>How Useful Is Old Information?</t>
+          <t>Structure-free model-based predictive signal control: A sensitivity analysis on a corridor with spillback</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
+          <t>Prediction errors ảnh hưởng MPC signal control ra sao?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
+          <t>Aimsun + MPC structure-free 4 nút; I reference biết demand ghi sẵn → II aggregation → III bias trên aggregation (§2.1, §2.2.4).</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
+          <t>Bias 1 đại lượng/lần (§3.3.1 tr15); Bảng 2 tr16 quét prediction 12/30/60 s và update 12/30/60 s; update ngắn bù một phần, state bias lớn làm mất bù (§3.3.2, §4).</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
+          <t>Không joint bias (§4 tr18); solver heuristic &lt;1% so full B&amp;B (Fig3d); metric delay/xe so reference, không regret/oracle D15. Hình chỉ đọc caption.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
+          <t>Traffic signals/MPC lặp; không suy D19Γ từ định tính.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>P/P/N</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -3715,22 +3934,22 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm code nguồn paper</t>
+          <t>Chưa kiểm</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>128 (Crossref, 2026-10-26)</t>
+          <t>4 (Crossref,2026-10-26)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>mitzenmacher2000oldinfo</t>
+          <t>poelman2023structurefree</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
+          <t>Tác giả đọc §2.2.4, §3.3, Bảng 2 nếu dùng cho nhãn PC2 ở L2.9; MT2/6/7 cập nhật ở follow-up.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -3747,42 +3966,42 @@
     <row r="19" ht="84" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
+          <t>Transient error approximation in a Lévy queue</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
+          <t>Stationary approximation gây sai số gì cho finite-horizon capacity allocation?</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
+          <t>Spectrally positive Lévy queue; transient expansion và correction staffing.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
+          <t>Eq2.4/2.7; Thm1 tr276, Prop4–5 tr282; terminal discussion journal§6 tr289.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
+          <t>AI-T, chưa proofs/replication; Lévy assumptions khác R2; §5.1 có u3 typo cần tránh chép.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
+          <t>Continuous capacity/average cost khác D21 randomness repair, one-shot routing regret.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>N/P/P</t>
+          <t>N/P/N</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -3792,22 +4011,22 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>117 (Crossref, 2026-10-26)</t>
+          <t>1 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>shaikh2001stale</t>
+          <t>mathijsen2017transient</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
+          <t>Tác giả đọc statement/§6; L2.7 kiểm decision geometry; A4/L2.9 còn mở.</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -3824,42 +4043,42 @@
     <row r="20" ht="84" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NDT1</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
+          <t>From Freshness to Effectiveness: Goal-Oriented Sampling for Remote Decision Making</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
+          <t>Khi nào lấy mẫu và chọn action để giảm remote-control cost dưới delay/rate constraint?</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
+          <t>Known-kernel finite controlled MDP; joint sampling/action, long-run average cost.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
+          <t>§III/Eq10 PDF5–7; §VII-D/Thm9/Cor2 PDF17: plateau theo allowed sampling budget.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
+          <t>AI-T v3; chưa proofs/replication/VoR full comparison. DOI TWC related thuộc bài khác.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
+          <t>Repeated joint policy khác D19 one-shot regret và D21 mean-rollout repair; solver ALP có trong §VII-C.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -3869,22 +4088,22 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa chạy code paper</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>185 (Crossref, 2026-10-25)</t>
+          <t>6 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>almasan2022ndt</t>
+          <t>li2026freshness</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
+          <t>Tác giả đọc §III tr5–6 (Problem1 Eq10) bản journal.</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -3894,49 +4113,49 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="21" ht="84" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>M00</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+          <t>How Useful Is Old Information?</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Phát hiện conflict giữa các SDN applications.</t>
+          <t>Load information cũ còn hữu ích khi dispatch jobs không?</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+          <t>Limiting ODE n→∞ + finite queue simulations; random/d-choice/shortest.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+          <t>§3.4 PDF10–12: shortest có thể thua random khi tin cũ; d2 hữu ích nhiều regime. §4 PDF19–21: random age giảm đồng bộ.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+          <t>AI-T submission, chưa VoR/full review/replication; d2 không luôn tốt nhất.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Conflict verdict khác expected decision regret của D18.</t>
+          <t>Sojourn time, repeated dispatch khác one-shot expected regret; chưa xác nhận controlled D21 ở phần đọc.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -3946,22 +4165,22 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Chưa kiểm</t>
+          <t>Chưa kiểm code nguồn paper</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>1 (Crossref, 2026-10-25)</t>
+          <t>128 (Crossref, 2026-10-26)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>polverini2026conflicts</t>
+          <t>mitzenmacher2000oldinfo</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+          <t>Tác giả đọc model/figures, giải thích herding; A4 kiểm re-solving, không claim GS&lt;0 mới.</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -3971,49 +4190,49 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="22" ht="84" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+          <t>Evaluating the Impact of Stale Link State on Quality-of-Service Routing</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Duy trì DT và kiểm candidate action xApp.</t>
+          <t>Stale link-state ảnh hưởng QoS routing và overhead thế nào?</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+          <t>Connection-level simulation; period/trigger/hold-down, topology, traffic và cost metric.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+          <t>§III/IV-A: blocking phụ thuộc update và topology; §V-A/Fig8: granularity phụ thuộc update policy; panel8b là setup failure.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+          <t>AI targeted, không replication; Fig8a tắt pruning,8b bật; không suy Γ.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+          <t>Blocking nhiều connection khác expected regret một action; C là metric resolution, không tự bằng D20 hoặc D21.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>P/P/N</t>
+          <t>N/P/P</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -4026,15 +4245,19 @@
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K22" s="2" t="n"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>117 (Crossref, 2026-10-26)</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>zhang2026opentwin</t>
+          <t>shaikh2001stale</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+          <t>Tác giả đọc §V-A/Fig8, giải thích E/M/R; M00 và Part2 để sau.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -4044,44 +4267,44 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
     <row r="23" ht="84" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>NDT1</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Value of Information in Feedback Control: Quantification</t>
+          <t>Network Digital Twin: Context, Enabling Technologies, and Opportunities</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+          <t>Twin hỗ trợ network modeling và tối ưu routing.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+          <t>GNN RouteNet-E ghép evolutionary optimizer.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+          <t>§II/IV, PDF2–5: KPI prediction và delay so shortest path; không là oracle D15.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>LQG, CE tối ưu, không có clipping.</t>
+          <t>Case study synthetic OMNeT++; input không phải backlog/mode D7.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Chỉ trục state; không có trục model.</t>
+          <t>Định vị NDT; chưa xác nhận2×2 can thiệp D20/D21.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -4101,17 +4324,17 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>75 (S2, 2026-10-24)</t>
+          <t>185 (Crossref, 2026-10-25)</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>soleymani2022value</t>
+          <t>almasan2022ndt</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+          <t>Tác giả mở §II, §IV và kiểm pipeline bằng lời mình.</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -4121,94 +4344,321 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
     <row r="24" ht="84" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Avoiding SDN Application Conflicts With Digital Twins: Design, Models and Proof of Concept</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Phát hiện conflict giữa các SDN applications.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>DTManager/Wrapper và4models; §III-A áp action ngay, feedback passive.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>§VI-A tr2047–2048: precision/recall cho4model; đã đọc text, chưa xem trực tiếp TableIII.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>PDF local403; hình/table chưa kiểm trực tiếp; input age chưa xác nhận.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Conflict verdict khác expected decision regret của D18.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1 (Crossref, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>polverini2026conflicts</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đọc §III-A/V/VI khi truy cập được nguồn; chưa cấp L-self.</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="84" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>OpenTwin: Closed-Loop Digital Twins for Trustworthy Policy Deployment in Open RAN</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Duy trì DT và kiểm candidate action xApp.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>§III/V/VI: calibrate outputs, resync inferred config, conformal gate.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>§VII-C Eq14: false approvals/tổng decision steps; §VIII-E tr11 dùng oracle biết outcome.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>AI targeted, chưa kiểm mọi theorem hoặc tái lập experiments.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Resync sửa config khác D20; safety/foresight benchmark khác D18/D15.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>zhang2026opentwin</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Tác giả đối chiếu §V-C/VI với D20/D21; giữ Gate pending.</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Value of Information in Feedback Control: Quantification</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Một gói thông tin cảm biến đáng giá bao nhiêu trong event-triggered control.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>VoI = chênh value function khi có/không truyền; LQG, controller CE.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Def.3 Eq.9 tr.6–7; Eq.22–24 tr.9: VoI là hàm của sai lệch ước lượng.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>LQG, CE tối ưu, không có clipping.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ trục state; không có trục model.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>P/P/N</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Mục liên quan</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Chưa kiểm</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>75 (S2, 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>soleymani2022value</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Part 2b (L2.6), cùng chương arXiv 2403.11926.</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>AI (chưa kiểm)</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>R34</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Optimal control of arrivals to queues with delayed queue length information</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Theo tiêu đề: điều khiển arrival khi thông tin chiều dài queue bị trễ.</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Chưa đọc.</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>CDC 1992 tr997–998: Thm2.1.2 JSEQ tối ưu với k=1; k≥2 có phản ví dụ (trỏ [4]); admission một queue: hai ngưỡng (Thm3.1.2).</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Chỉ bản hội nghị 2 trang, chứng minh lược; mô hình đúng (không trục model).</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Chưa đánh giá.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>P/P/P</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Metadata</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Chưa kiểm</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>34 (Crossref, 2026-10-24)</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>kuri1995optimal</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Cần bản TAC 40(8) 1995.</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>AI (chưa kiểm)</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O24"/>
+  <autoFilter ref="A1:O27"/>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Thứ cấp,Metadata,Abstract,Mục liên quan,Full bài"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"AI (chưa kiểm),Tôi"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4250,7 +4700,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>23 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
+          <t>26 nguồn trong catalog hiện dùng; xem cột Vai trò hiện tại. Không phải danh sách đầy đủ về NDT hay bài tập phải đọc hết.</t>
         </is>
       </c>
     </row>

</xml_diff>